<commit_message>
lógica de cálculo vgvs
</commit_message>
<xml_diff>
--- a/areas_land_bank_com_id.xlsx
+++ b/areas_land_bank_com_id.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="EsteLivro" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Departamento Controladoria\3 - BT 360º\Landbank\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinicius.castro\Documents\01 Profissional\Buriti Empreendimentos\Repositórios\land-bank-mapa-brasil-terrenos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2629E1CF-09DD-4F32-A64D-AB17E500600A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5256DE6A-6317-4F17-9C7A-ABDC3532BCF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="960" windowWidth="29040" windowHeight="15720" xr2:uid="{2D7381EB-1656-47BB-A82F-14AB3B13CCCD}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2D7381EB-1656-47BB-A82F-14AB3B13CCCD}"/>
   </bookViews>
   <sheets>
     <sheet name="AREAS" sheetId="1" r:id="rId1"/>
@@ -5306,7 +5306,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2192" uniqueCount="737">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2195" uniqueCount="737">
   <si>
     <t>Nome</t>
   </si>
@@ -7529,17 +7529,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="11">
-    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="0.0%_);\(0.0%\);0.0%_);@_)"/>
-    <numFmt numFmtId="165" formatCode="0.00%_);\(0.00%\);0.00%_);@_)"/>
-    <numFmt numFmtId="166" formatCode="0%_);\(0%\);0%_);@_)"/>
-    <numFmt numFmtId="167" formatCode="[$-416]mmm\-yy;@"/>
-    <numFmt numFmtId="168" formatCode="&quot;Ativo&quot;;\-#,##0;[Red]&quot;Inativo&quot;"/>
-    <numFmt numFmtId="169" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="170" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="171" formatCode="0.0%"/>
-    <numFmt numFmtId="172" formatCode="#,##0.00&quot;x&quot;"/>
+    <numFmt numFmtId="164" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="0.0%_);\(0.0%\);0.0%_);@_)"/>
+    <numFmt numFmtId="167" formatCode="0.00%_);\(0.00%\);0.00%_);@_)"/>
+    <numFmt numFmtId="168" formatCode="0%_);\(0%\);0%_);@_)"/>
+    <numFmt numFmtId="169" formatCode="[$-416]mmm\-yy;@"/>
+    <numFmt numFmtId="170" formatCode="&quot;Ativo&quot;;\-#,##0;[Red]&quot;Inativo&quot;"/>
+    <numFmt numFmtId="171" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="172" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="173" formatCode="0.0%"/>
+    <numFmt numFmtId="174" formatCode="#,##0.00&quot;x&quot;"/>
   </numFmts>
   <fonts count="16" x14ac:knownFonts="1">
     <font>
@@ -7866,11 +7866,11 @@
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -7893,25 +7893,25 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="37" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -7923,19 +7923,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="3" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="3" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="3" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -7944,10 +7944,10 @@
     <xf numFmtId="37" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="3" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="4" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -7959,37 +7959,37 @@
     <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="4" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="37" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="37" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="3" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="3" fillId="3" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -7998,49 +7998,49 @@
     <xf numFmtId="49" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="3" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="4" fillId="3" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="37" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="37" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="3" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="3" fillId="3" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="37" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="6" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="3" fillId="6" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="3" fillId="3" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="3" fillId="3" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -8049,13 +8049,13 @@
     <xf numFmtId="37" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="8" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="4" fillId="8" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="37" fontId="3" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="8" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="4" fillId="8" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -8068,34 +8068,34 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="174" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="37" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="3" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="44" fontId="1" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="3" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="3" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="170" fontId="4" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="172" fontId="4" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -8132,7 +8132,7 @@
     <xf numFmtId="0" fontId="11" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="12" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -8157,8 +8157,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="11" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -8169,13 +8168,13 @@
     <xf numFmtId="10" fontId="11" fillId="3" borderId="12" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="11" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
-    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hiperligação" xfId="1" builtinId="8"/>
     <cellStyle name="Moeda" xfId="3" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Porcentagem" xfId="4" builtinId="5"/>
+    <cellStyle name="Percentagem" xfId="4" builtinId="5"/>
     <cellStyle name="Vírgula" xfId="2" builtinId="3"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -8196,10 +8195,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8521,49 +8516,49 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BB1E7F9-B7E0-4EE5-A96E-08F27078CA81}">
   <sheetPr codeName="Folha1"/>
   <dimension ref="A1:AP241"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.26953125" customWidth="1"/>
-    <col min="2" max="2" width="58.453125" style="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="4" max="4" width="22.453125" customWidth="1" collapsed="1"/>
-    <col min="5" max="5" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="10.54296875" customWidth="1"/>
-    <col min="10" max="10" width="11.81640625" customWidth="1"/>
-    <col min="11" max="11" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="28.6328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="26.26953125" style="77" customWidth="1"/>
-    <col min="14" max="14" width="53.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.08984375" style="27" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.26953125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.81640625" customWidth="1"/>
-    <col min="20" max="20" width="11.54296875" customWidth="1"/>
-    <col min="21" max="21" width="11.26953125" customWidth="1"/>
+    <col min="1" max="1" width="15.21875" customWidth="1"/>
+    <col min="2" max="2" width="58.44140625" style="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.77734375" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="4" max="4" width="22.44140625" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="10.5546875" customWidth="1"/>
+    <col min="10" max="10" width="11.77734375" customWidth="1"/>
+    <col min="11" max="11" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="26.21875" style="77" customWidth="1"/>
+    <col min="14" max="14" width="53.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.109375" style="27" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.77734375" customWidth="1"/>
+    <col min="20" max="20" width="11.5546875" customWidth="1"/>
+    <col min="21" max="21" width="11.21875" customWidth="1"/>
     <col min="22" max="22" width="14" customWidth="1"/>
-    <col min="23" max="23" width="10.26953125" customWidth="1"/>
-    <col min="24" max="24" width="10.81640625" customWidth="1"/>
-    <col min="25" max="25" width="12.7265625" customWidth="1"/>
+    <col min="23" max="23" width="10.21875" customWidth="1"/>
+    <col min="24" max="24" width="10.77734375" customWidth="1"/>
+    <col min="25" max="25" width="12.77734375" customWidth="1"/>
     <col min="26" max="26" width="12" customWidth="1"/>
-    <col min="27" max="27" width="11.54296875" customWidth="1"/>
-    <col min="28" max="28" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="11.81640625" customWidth="1"/>
-    <col min="31" max="31" width="11.1796875" customWidth="1"/>
-    <col min="32" max="32" width="12.26953125" customWidth="1"/>
-    <col min="33" max="33" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.54296875" customWidth="1"/>
+    <col min="27" max="27" width="11.5546875" customWidth="1"/>
+    <col min="28" max="28" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11.77734375" customWidth="1"/>
+    <col min="31" max="31" width="11.21875" customWidth="1"/>
+    <col min="32" max="32" width="12.21875" customWidth="1"/>
+    <col min="33" max="33" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.5546875" customWidth="1"/>
     <col min="37" max="38" width="9" customWidth="1"/>
     <col min="39" max="39" width="16" bestFit="1" customWidth="1"/>
-    <col min="40" max="41" width="12.81640625" customWidth="1"/>
-    <col min="42" max="42" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="40" max="41" width="12.77734375" customWidth="1"/>
+    <col min="42" max="42" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" ht="52" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:42" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>568</v>
       </c>
@@ -8691,7 +8686,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="2" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
         <v>576</v>
       </c>
@@ -8810,7 +8805,7 @@
         <v>3.3809797786673061</v>
       </c>
     </row>
-    <row r="3" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A3" s="64" t="s">
         <v>577</v>
       </c>
@@ -8931,7 +8926,7 @@
         <v>4.8097271922736544</v>
       </c>
     </row>
-    <row r="4" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A4" s="64" t="s">
         <v>577</v>
       </c>
@@ -9052,7 +9047,7 @@
         <v>5.3580126643935699</v>
       </c>
     </row>
-    <row r="5" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="64" t="s">
         <v>578</v>
       </c>
@@ -9171,7 +9166,7 @@
         <v>4.5078888054094666</v>
       </c>
     </row>
-    <row r="6" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="64" t="s">
         <v>579</v>
       </c>
@@ -9290,7 +9285,7 @@
         <v>4.5078888054094675</v>
       </c>
     </row>
-    <row r="7" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A7" s="64" t="s">
         <v>579</v>
       </c>
@@ -9409,7 +9404,7 @@
         <v>4.5078888054094666</v>
       </c>
     </row>
-    <row r="8" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A8" s="64" t="s">
         <v>579</v>
       </c>
@@ -9528,7 +9523,7 @@
         <v>4.5078888054094683</v>
       </c>
     </row>
-    <row r="9" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A9" s="64" t="s">
         <v>579</v>
       </c>
@@ -9647,7 +9642,7 @@
         <v>4.5078888054094683</v>
       </c>
     </row>
-    <row r="10" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A10" s="64" t="s">
         <v>579</v>
       </c>
@@ -9766,7 +9761,7 @@
         <v>4.5078888054094683</v>
       </c>
     </row>
-    <row r="11" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A11" s="64" t="s">
         <v>570</v>
       </c>
@@ -9883,7 +9878,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="12" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A12" s="64" t="s">
         <v>571</v>
       </c>
@@ -10000,7 +9995,7 @@
         <v>3.2306536438767841</v>
       </c>
     </row>
-    <row r="13" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A13" s="64" t="s">
         <v>572</v>
       </c>
@@ -10117,7 +10112,7 @@
         <v>4.883546205860255</v>
       </c>
     </row>
-    <row r="14" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A14" s="64" t="s">
         <v>572</v>
       </c>
@@ -10234,7 +10229,7 @@
         <v>4.883546205860255</v>
       </c>
     </row>
-    <row r="15" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A15" s="64" t="s">
         <v>573</v>
       </c>
@@ -10351,7 +10346,7 @@
         <v>3.7565740045078888</v>
       </c>
     </row>
-    <row r="16" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A16" s="64" t="s">
         <v>574</v>
       </c>
@@ -10468,7 +10463,7 @@
         <v>3.7565740045078897</v>
       </c>
     </row>
-    <row r="17" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A17" s="64" t="s">
         <v>575</v>
       </c>
@@ -10585,7 +10580,7 @@
         <v>3.7565740045078893</v>
       </c>
     </row>
-    <row r="18" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A18" s="64" t="s">
         <v>580</v>
       </c>
@@ -10702,7 +10697,7 @@
         <v>3.230653643876785</v>
       </c>
     </row>
-    <row r="19" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A19" s="64" t="s">
         <v>581</v>
       </c>
@@ -10819,7 +10814,7 @@
         <v>2.9301277235161534</v>
       </c>
     </row>
-    <row r="20" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A20" s="64" t="s">
         <v>581</v>
       </c>
@@ -10936,7 +10931,7 @@
         <v>2.9301277235161534</v>
       </c>
     </row>
-    <row r="21" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A21" s="64" t="s">
         <v>581</v>
       </c>
@@ -11053,7 +11048,7 @@
         <v>2.9301277235161534</v>
       </c>
     </row>
-    <row r="22" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A22" s="64" t="s">
         <v>581</v>
       </c>
@@ -11170,7 +11165,7 @@
         <v>2.9301277235161534</v>
       </c>
     </row>
-    <row r="23" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A23" s="64" t="s">
         <v>581</v>
       </c>
@@ -11287,7 +11282,7 @@
         <v>2.9301277235161534</v>
       </c>
     </row>
-    <row r="24" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A24" s="64" t="s">
         <v>581</v>
       </c>
@@ -11404,7 +11399,7 @@
         <v>2.9301277235161534</v>
       </c>
     </row>
-    <row r="25" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A25" s="64" t="s">
         <v>581</v>
       </c>
@@ -11521,7 +11516,7 @@
         <v>2.9301277235161534</v>
       </c>
     </row>
-    <row r="26" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A26" s="64" t="s">
         <v>582</v>
       </c>
@@ -11640,7 +11635,7 @@
         <v>0.83115017886351839</v>
       </c>
     </row>
-    <row r="27" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A27" s="64" t="s">
         <v>583</v>
       </c>
@@ -11757,7 +11752,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="28" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A28" s="64" t="s">
         <v>583</v>
       </c>
@@ -11873,7 +11868,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="29" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A29" s="64" t="s">
         <v>583</v>
       </c>
@@ -11990,7 +11985,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="30" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A30" s="64" t="s">
         <v>583</v>
       </c>
@@ -12107,7 +12102,7 @@
         <v>4.140625</v>
       </c>
     </row>
-    <row r="31" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A31" s="64" t="s">
         <v>583</v>
       </c>
@@ -12224,7 +12219,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="32" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A32" s="64" t="s">
         <v>583</v>
       </c>
@@ -12341,7 +12336,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="33" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A33" s="64" t="s">
         <v>583</v>
       </c>
@@ -12458,7 +12453,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="34" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A34" s="64" t="s">
         <v>583</v>
       </c>
@@ -12575,7 +12570,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="35" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A35" s="64" t="s">
         <v>583</v>
       </c>
@@ -12692,7 +12687,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="36" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A36" s="64" t="s">
         <v>583</v>
       </c>
@@ -12809,7 +12804,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="37" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A37" s="64" t="s">
         <v>583</v>
       </c>
@@ -12926,7 +12921,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="38" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A38" s="64" t="s">
         <v>583</v>
       </c>
@@ -13043,7 +13038,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="39" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A39" s="64" t="s">
         <v>583</v>
       </c>
@@ -13160,7 +13155,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="40" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A40" s="64" t="s">
         <v>583</v>
       </c>
@@ -13277,7 +13272,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="41" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A41" s="64" t="s">
         <v>583</v>
       </c>
@@ -13394,7 +13389,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="42" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A42" s="64" t="s">
         <v>583</v>
       </c>
@@ -13511,7 +13506,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="43" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A43" s="64" t="s">
         <v>583</v>
       </c>
@@ -13628,7 +13623,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="44" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A44" s="64" t="s">
         <v>583</v>
       </c>
@@ -13745,7 +13740,7 @@
         <v>4.296875</v>
       </c>
     </row>
-    <row r="45" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A45" s="64" t="s">
         <v>583</v>
       </c>
@@ -13862,7 +13857,7 @@
         <v>3.90625</v>
       </c>
     </row>
-    <row r="46" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A46" s="64" t="s">
         <v>584</v>
       </c>
@@ -13985,7 +13980,7 @@
         <v>1.5033333068541384</v>
       </c>
     </row>
-    <row r="47" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A47" s="64" t="s">
         <v>584</v>
       </c>
@@ -14108,7 +14103,7 @@
         <v>1.5033333068541381</v>
       </c>
     </row>
-    <row r="48" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A48" s="64" t="s">
         <v>584</v>
       </c>
@@ -14231,7 +14226,7 @@
         <v>1.1881369949110563</v>
       </c>
     </row>
-    <row r="49" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A49" s="64" t="s">
         <v>584</v>
       </c>
@@ -14354,7 +14349,7 @@
         <v>1.1629101414416052</v>
       </c>
     </row>
-    <row r="50" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A50" s="64" t="s">
         <v>585</v>
       </c>
@@ -14470,7 +14465,7 @@
         <v>3.9062500000000004</v>
       </c>
     </row>
-    <row r="51" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A51" s="64" t="s">
         <v>587</v>
       </c>
@@ -14587,7 +14582,7 @@
         <v>4.6875000000000009</v>
       </c>
     </row>
-    <row r="52" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A52" s="64" t="s">
         <v>681</v>
       </c>
@@ -14704,7 +14699,7 @@
         <v>3.2407407407407409</v>
       </c>
     </row>
-    <row r="53" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A53" s="64" t="s">
         <v>586</v>
       </c>
@@ -14821,7 +14816,7 @@
         <v>3.2407407407407409</v>
       </c>
     </row>
-    <row r="54" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A54" s="64" t="s">
         <v>588</v>
       </c>
@@ -14938,7 +14933,7 @@
         <v>6.2499999999999991</v>
       </c>
     </row>
-    <row r="55" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A55" s="64" t="s">
         <v>589</v>
       </c>
@@ -15056,7 +15051,7 @@
         <v>3.7037037037037033</v>
       </c>
     </row>
-    <row r="56" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A56" s="64" t="s">
         <v>591</v>
       </c>
@@ -15181,7 +15176,7 @@
         <v>2.0794444816235882</v>
       </c>
     </row>
-    <row r="57" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A57" s="64" t="s">
         <v>591</v>
       </c>
@@ -15305,7 +15300,7 @@
         <v>0.682062825375507</v>
       </c>
     </row>
-    <row r="58" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A58" s="64" t="s">
         <v>590</v>
       </c>
@@ -15428,7 +15423,7 @@
         <v>1.584067227618178</v>
       </c>
     </row>
-    <row r="59" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A59" s="64" t="s">
         <v>592</v>
       </c>
@@ -15551,7 +15546,7 @@
         <v>1.2626874796242238</v>
       </c>
     </row>
-    <row r="60" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A60" s="64" t="s">
         <v>593</v>
       </c>
@@ -15674,7 +15669,7 @@
         <v>1.165542478997921</v>
       </c>
     </row>
-    <row r="61" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A61" s="64" t="s">
         <v>593</v>
       </c>
@@ -15797,7 +15792,7 @@
         <v>1.1453025708336924</v>
       </c>
     </row>
-    <row r="62" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A62" s="64" t="s">
         <v>594</v>
       </c>
@@ -15920,7 +15915,7 @@
         <v>1.0499523822058021</v>
       </c>
     </row>
-    <row r="63" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A63" s="64" t="s">
         <v>595</v>
       </c>
@@ -16037,7 +16032,7 @@
         <v>3.9384920139218527</v>
       </c>
     </row>
-    <row r="64" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A64" s="64" t="s">
         <v>595</v>
       </c>
@@ -16154,7 +16149,7 @@
         <v>3.9384920139218527</v>
       </c>
     </row>
-    <row r="65" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A65" s="64" t="s">
         <v>595</v>
       </c>
@@ -16271,7 +16266,7 @@
         <v>3.9384920139218527</v>
       </c>
     </row>
-    <row r="66" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A66" s="64" t="s">
         <v>596</v>
       </c>
@@ -16390,7 +16385,7 @@
         <v>3.5833333333333335</v>
       </c>
     </row>
-    <row r="67" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A67" s="64" t="s">
         <v>597</v>
       </c>
@@ -16509,7 +16504,7 @@
         <v>3.8333333333333335</v>
       </c>
     </row>
-    <row r="68" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A68" s="64" t="s">
         <v>598</v>
       </c>
@@ -16628,7 +16623,7 @@
         <v>3.5833333333333335</v>
       </c>
     </row>
-    <row r="69" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A69" s="64" t="s">
         <v>598</v>
       </c>
@@ -16747,7 +16742,7 @@
         <v>3.5833333333333335</v>
       </c>
     </row>
-    <row r="70" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A70" s="64" t="s">
         <v>599</v>
       </c>
@@ -16871,7 +16866,7 @@
         <v>1.6840907460634127</v>
       </c>
     </row>
-    <row r="71" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A71" s="64" t="s">
         <v>600</v>
       </c>
@@ -16995,7 +16990,7 @@
         <v>1.7104564330775569</v>
       </c>
     </row>
-    <row r="72" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A72" s="64" t="s">
         <v>600</v>
       </c>
@@ -17119,7 +17114,7 @@
         <v>1.6579735962048303</v>
       </c>
     </row>
-    <row r="73" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A73" s="64" t="s">
         <v>601</v>
       </c>
@@ -17241,7 +17236,7 @@
         <v>2.5287610566591523</v>
       </c>
     </row>
-    <row r="74" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A74" s="64" t="s">
         <v>601</v>
       </c>
@@ -17363,7 +17358,7 @@
         <v>2.4793535855822042</v>
       </c>
     </row>
-    <row r="75" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A75" s="64" t="s">
         <v>602</v>
       </c>
@@ -17488,7 +17483,7 @@
         <v>1.890388055872956</v>
       </c>
     </row>
-    <row r="76" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A76" s="64" t="s">
         <v>602</v>
       </c>
@@ -17613,7 +17608,7 @@
         <v>1.8605083275965164</v>
       </c>
     </row>
-    <row r="77" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A77" s="64" t="s">
         <v>603</v>
       </c>
@@ -17738,7 +17733,7 @@
         <v>1.8523399895648596</v>
       </c>
     </row>
-    <row r="78" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A78" s="64" t="s">
         <v>603</v>
       </c>
@@ -17863,7 +17858,7 @@
         <v>1.7669888872138106</v>
       </c>
     </row>
-    <row r="79" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A79" s="64" t="s">
         <v>604</v>
       </c>
@@ -17986,7 +17981,7 @@
         <v>0.64100515446669049</v>
       </c>
     </row>
-    <row r="80" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A80" s="64" t="s">
         <v>604</v>
       </c>
@@ -18109,7 +18104,7 @@
         <v>0.62670976763932151</v>
       </c>
     </row>
-    <row r="81" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A81" s="64" t="s">
         <v>605</v>
       </c>
@@ -18232,7 +18227,7 @@
         <v>0.76883870310314895</v>
       </c>
     </row>
-    <row r="82" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A82" s="64" t="s">
         <v>606</v>
       </c>
@@ -18355,7 +18350,7 @@
         <v>1.4269848890125221</v>
       </c>
     </row>
-    <row r="83" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A83" s="64" t="s">
         <v>607</v>
       </c>
@@ -18478,7 +18473,7 @@
         <v>0.83525452781953513</v>
       </c>
     </row>
-    <row r="84" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A84" s="64" t="s">
         <v>607</v>
       </c>
@@ -18601,7 +18596,7 @@
         <v>0.81799598953212038</v>
       </c>
     </row>
-    <row r="85" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A85" s="64" t="s">
         <v>607</v>
       </c>
@@ -18724,7 +18719,7 @@
         <v>0.78388138912123639</v>
       </c>
     </row>
-    <row r="86" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A86" s="64" t="s">
         <v>608</v>
       </c>
@@ -18847,7 +18842,7 @@
         <v>1.1501266268686077</v>
       </c>
     </row>
-    <row r="87" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A87" s="64" t="s">
         <v>609</v>
       </c>
@@ -18972,7 +18967,7 @@
         <v>0.23299756298435631</v>
       </c>
     </row>
-    <row r="88" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A88" s="64" t="s">
         <v>609</v>
       </c>
@@ -19097,7 +19092,7 @@
         <v>1.2387943662501089</v>
       </c>
     </row>
-    <row r="89" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A89" s="64" t="s">
         <v>610</v>
       </c>
@@ -19220,7 +19215,7 @@
         <v>1.5149909654595908</v>
       </c>
     </row>
-    <row r="90" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A90" s="64" t="s">
         <v>682</v>
       </c>
@@ -19343,7 +19338,7 @@
         <v>1.2046020634661616</v>
       </c>
     </row>
-    <row r="91" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A91" s="64" t="s">
         <v>611</v>
       </c>
@@ -19466,7 +19461,7 @@
         <v>1.2072988815514583</v>
       </c>
     </row>
-    <row r="92" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A92" s="64" t="s">
         <v>611</v>
       </c>
@@ -19589,7 +19584,7 @@
         <v>1.4090811331942312</v>
       </c>
     </row>
-    <row r="93" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A93" s="64" t="s">
         <v>611</v>
       </c>
@@ -19712,7 +19707,7 @@
         <v>1.1397336017719824</v>
       </c>
     </row>
-    <row r="94" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A94" s="64" t="s">
         <v>611</v>
       </c>
@@ -19835,7 +19830,7 @@
         <v>1.0959959051299162</v>
       </c>
     </row>
-    <row r="95" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A95" s="64" t="s">
         <v>611</v>
       </c>
@@ -19958,7 +19953,7 @@
         <v>1.0527200029561115</v>
       </c>
     </row>
-    <row r="96" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A96" s="64" t="s">
         <v>612</v>
       </c>
@@ -20083,7 +20078,7 @@
         <v>2.1202973983797322</v>
       </c>
     </row>
-    <row r="97" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A97" s="64" t="s">
         <v>613</v>
       </c>
@@ -20208,7 +20203,7 @@
         <v>2.0772596632135061</v>
       </c>
     </row>
-    <row r="98" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A98" s="64" t="s">
         <v>615</v>
       </c>
@@ -20331,7 +20326,7 @@
         <v>1.5361651825388483</v>
       </c>
     </row>
-    <row r="99" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A99" s="64" t="s">
         <v>615</v>
       </c>
@@ -20454,7 +20449,7 @@
         <v>1.5065784699927574</v>
       </c>
     </row>
-    <row r="100" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A100" s="64" t="s">
         <v>615</v>
       </c>
@@ -20577,7 +20572,7 @@
         <v>1.4478450040383797</v>
       </c>
     </row>
-    <row r="101" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A101" s="64" t="s">
         <v>614</v>
       </c>
@@ -20700,7 +20695,7 @@
         <v>1.0994472988394468</v>
       </c>
     </row>
-    <row r="102" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A102" s="64" t="s">
         <v>614</v>
       </c>
@@ -20823,7 +20818,7 @@
         <v>1.0586916755795146</v>
       </c>
     </row>
-    <row r="103" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A103" s="64" t="s">
         <v>616</v>
       </c>
@@ -20946,7 +20941,7 @@
         <v>1.6691380981214541</v>
       </c>
     </row>
-    <row r="104" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A104" s="64" t="s">
         <v>616</v>
       </c>
@@ -21069,7 +21064,7 @@
         <v>1.6065963825333243</v>
       </c>
     </row>
-    <row r="105" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A105" s="64" t="s">
         <v>617</v>
       </c>
@@ -21192,7 +21187,7 @@
         <v>0.90690345120653837</v>
       </c>
     </row>
-    <row r="106" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A106" s="64" t="s">
         <v>618</v>
       </c>
@@ -21315,7 +21310,7 @@
         <v>0.87259450365707092</v>
       </c>
     </row>
-    <row r="107" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A107" s="64" t="s">
         <v>619</v>
       </c>
@@ -21438,7 +21433,7 @@
         <v>0.83860953776262182</v>
       </c>
     </row>
-    <row r="108" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A108" s="64" t="s">
         <v>619</v>
       </c>
@@ -21561,7 +21556,7 @@
         <v>0.80502313984963059</v>
       </c>
     </row>
-    <row r="109" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A109" s="64" t="s">
         <v>619</v>
       </c>
@@ -21684,7 +21679,7 @@
         <v>2.024472392638037</v>
       </c>
     </row>
-    <row r="110" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A110" s="64" t="s">
         <v>619</v>
       </c>
@@ -21807,7 +21802,7 @@
         <v>2.024472392638037</v>
       </c>
     </row>
-    <row r="111" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A111" s="64" t="s">
         <v>619</v>
       </c>
@@ -21930,7 +21925,7 @@
         <v>2.024472392638037</v>
       </c>
     </row>
-    <row r="112" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A112" s="64" t="s">
         <v>619</v>
       </c>
@@ -22053,7 +22048,7 @@
         <v>2.024472392638037</v>
       </c>
     </row>
-    <row r="113" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A113" s="64" t="s">
         <v>619</v>
       </c>
@@ -22176,7 +22171,7 @@
         <v>2.024472392638037</v>
       </c>
     </row>
-    <row r="114" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A114" s="64" t="s">
         <v>620</v>
       </c>
@@ -22299,7 +22294,7 @@
         <v>0.73245167478536033</v>
       </c>
     </row>
-    <row r="115" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A115" s="64" t="s">
         <v>621</v>
       </c>
@@ -22422,7 +22417,7 @@
         <v>0.70127185350915722</v>
       </c>
     </row>
-    <row r="116" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A116" s="64" t="s">
         <v>621</v>
       </c>
@@ -22545,7 +22540,7 @@
         <v>0.6706877524292354</v>
       </c>
     </row>
-    <row r="117" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A117" s="64" t="s">
         <v>621</v>
       </c>
@@ -22668,7 +22663,7 @@
         <v>0.64075267145675929</v>
       </c>
     </row>
-    <row r="118" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A118" s="64" t="s">
         <v>621</v>
       </c>
@@ -22791,7 +22786,7 @@
         <v>0.61151467271213211</v>
       </c>
     </row>
-    <row r="119" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A119" s="64" t="s">
         <v>621</v>
       </c>
@@ -22914,7 +22909,7 @@
         <v>1.9492775508164899</v>
       </c>
     </row>
-    <row r="120" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A120" s="64" t="s">
         <v>622</v>
       </c>
@@ -23037,7 +23032,7 @@
         <v>1.2292115404911319</v>
       </c>
     </row>
-    <row r="121" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A121" s="64" t="s">
         <v>623</v>
       </c>
@@ -23160,7 +23155,7 @@
         <v>1.2413630323963301</v>
       </c>
     </row>
-    <row r="122" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A122" s="64" t="s">
         <v>624</v>
       </c>
@@ -23283,7 +23278,7 @@
         <v>1.2561653093904881</v>
       </c>
     </row>
-    <row r="123" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A123" s="64" t="s">
         <v>625</v>
       </c>
@@ -23406,7 +23401,7 @@
         <v>1.2113560025023844</v>
       </c>
     </row>
-    <row r="124" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A124" s="64" t="s">
         <v>626</v>
       </c>
@@ -23529,7 +23524,7 @@
         <v>2.613496932515337</v>
       </c>
     </row>
-    <row r="125" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A125" s="64" t="s">
         <v>626</v>
       </c>
@@ -23652,7 +23647,7 @@
         <v>2.6134969325153379</v>
       </c>
     </row>
-    <row r="126" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A126" s="64" t="s">
         <v>627</v>
       </c>
@@ -23775,7 +23770,7 @@
         <v>1.3821716627734322</v>
       </c>
     </row>
-    <row r="127" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A127" s="64" t="s">
         <v>628</v>
       </c>
@@ -23898,7 +23893,7 @@
         <v>1.3508286832235206</v>
       </c>
     </row>
-    <row r="128" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A128" s="64" t="s">
         <v>628</v>
       </c>
@@ -24021,7 +24016,7 @@
         <v>1.3273996567144928</v>
       </c>
     </row>
-    <row r="129" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A129" s="64" t="s">
         <v>629</v>
       </c>
@@ -24144,7 +24139,7 @@
         <v>1.1478379123898736</v>
       </c>
     </row>
-    <row r="130" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A130" s="64" t="s">
         <v>630</v>
       </c>
@@ -24267,7 +24262,7 @@
         <v>1.1873209657838852</v>
       </c>
     </row>
-    <row r="131" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A131" s="64" t="s">
         <v>630</v>
       </c>
@@ -24390,7 +24385,7 @@
         <v>1.1478379123898732</v>
       </c>
     </row>
-    <row r="132" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A132" s="64" t="s">
         <v>631</v>
       </c>
@@ -24513,7 +24508,7 @@
         <v>1.1697737528257561</v>
       </c>
     </row>
-    <row r="133" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A133" s="64" t="s">
         <v>632</v>
       </c>
@@ -24636,7 +24631,7 @@
         <v>1.1478379123898734</v>
       </c>
     </row>
-    <row r="134" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A134" s="64" t="s">
         <v>633</v>
       </c>
@@ -24759,7 +24754,7 @@
         <v>1.1917791466511929</v>
       </c>
     </row>
-    <row r="135" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A135" s="64" t="s">
         <v>633</v>
       </c>
@@ -24882,7 +24877,7 @@
         <v>1.1697737528257561</v>
       </c>
     </row>
-    <row r="136" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A136" s="64" t="s">
         <v>633</v>
       </c>
@@ -25005,7 +25000,7 @@
         <v>1.1478379123898732</v>
       </c>
     </row>
-    <row r="137" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A137" s="64" t="s">
         <v>634</v>
       </c>
@@ -25127,7 +25122,7 @@
         <v>1.100201380402013</v>
       </c>
     </row>
-    <row r="138" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A138" s="64" t="s">
         <v>634</v>
       </c>
@@ -25244,7 +25239,7 @@
         <v>3.4285714285714284</v>
       </c>
     </row>
-    <row r="139" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A139" s="64" t="s">
         <v>634</v>
       </c>
@@ -25366,7 +25361,7 @@
         <v>1.5534532233799874</v>
       </c>
     </row>
-    <row r="140" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A140" s="64" t="s">
         <v>634</v>
       </c>
@@ -25483,7 +25478,7 @@
         <v>3.4285714285714284</v>
       </c>
     </row>
-    <row r="141" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A141" s="64" t="s">
         <v>635</v>
       </c>
@@ -25606,7 +25601,7 @@
         <v>1.3402722285622568</v>
       </c>
     </row>
-    <row r="142" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A142" s="64" t="s">
         <v>635</v>
       </c>
@@ -25729,7 +25724,7 @@
         <v>1.1069472501692708</v>
       </c>
     </row>
-    <row r="143" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A143" s="64" t="s">
         <v>635</v>
       </c>
@@ -25852,7 +25847,7 @@
         <v>1.3096934841312509</v>
       </c>
     </row>
-    <row r="144" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A144" s="64" t="s">
         <v>636</v>
       </c>
@@ -25975,7 +25970,7 @@
         <v>1.2649802836537249</v>
       </c>
     </row>
-    <row r="145" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A145" s="64" t="s">
         <v>637</v>
       </c>
@@ -26098,7 +26093,7 @@
         <v>1.242648133063637</v>
       </c>
     </row>
-    <row r="146" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A146" s="64" t="s">
         <v>638</v>
       </c>
@@ -26221,7 +26216,7 @@
         <v>0.90074899958421728</v>
       </c>
     </row>
-    <row r="147" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A147" s="64" t="s">
         <v>638</v>
       </c>
@@ -26344,7 +26339,7 @@
         <v>0.86471997316517379</v>
       </c>
     </row>
-    <row r="148" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A148" s="64" t="s">
         <v>638</v>
       </c>
@@ -26467,7 +26462,7 @@
         <v>0.8291908931927453</v>
       </c>
     </row>
-    <row r="149" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A149" s="64" t="s">
         <v>638</v>
       </c>
@@ -26590,7 +26585,7 @@
         <v>0.82391222601076908</v>
       </c>
     </row>
-    <row r="150" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A150" s="64" t="s">
         <v>638</v>
       </c>
@@ -26713,7 +26708,7 @@
         <v>1.307592918802565</v>
       </c>
     </row>
-    <row r="151" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A151" s="64" t="s">
         <v>638</v>
       </c>
@@ -26836,7 +26831,7 @@
         <v>1.259710619839457</v>
       </c>
     </row>
-    <row r="152" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A152" s="64" t="s">
         <v>638</v>
       </c>
@@ -26953,7 +26948,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="153" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A153" s="64" t="s">
         <v>638</v>
       </c>
@@ -27076,7 +27071,7 @@
         <v>1.5199940748831153</v>
       </c>
     </row>
-    <row r="154" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A154" s="64" t="s">
         <v>638</v>
       </c>
@@ -27199,7 +27194,7 @@
         <v>0.94841385595929528</v>
       </c>
     </row>
-    <row r="155" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A155" s="64" t="s">
         <v>639</v>
       </c>
@@ -27322,7 +27317,7 @@
         <v>2.001711919813113</v>
       </c>
     </row>
-    <row r="156" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A156" s="64" t="s">
         <v>639</v>
       </c>
@@ -27445,7 +27440,7 @@
         <v>2.7873981870831179</v>
       </c>
     </row>
-    <row r="157" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A157" s="64" t="s">
         <v>639</v>
       </c>
@@ -27568,7 +27563,7 @@
         <v>1.8835744163813872</v>
       </c>
     </row>
-    <row r="158" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A158" s="64" t="s">
         <v>684</v>
       </c>
@@ -27691,7 +27686,7 @@
         <v>1.3178084967631456</v>
       </c>
     </row>
-    <row r="159" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A159" s="64" t="s">
         <v>683</v>
       </c>
@@ -27814,7 +27809,7 @@
         <v>1.3730404099510281</v>
       </c>
     </row>
-    <row r="160" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A160" s="64" t="s">
         <v>640</v>
       </c>
@@ -27937,7 +27932,7 @@
         <v>1.3848749369337743</v>
       </c>
     </row>
-    <row r="161" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A161" s="64" t="s">
         <v>641</v>
       </c>
@@ -28060,7 +28055,7 @@
         <v>1.3585676614027813</v>
       </c>
     </row>
-    <row r="162" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A162" s="64" t="s">
         <v>642</v>
       </c>
@@ -28183,7 +28178,7 @@
         <v>1.372740519264412</v>
       </c>
     </row>
-    <row r="163" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A163" s="64" t="s">
         <v>643</v>
       </c>
@@ -28306,7 +28301,7 @@
         <v>1.3209122633460484</v>
       </c>
     </row>
-    <row r="164" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A164" s="64" t="s">
         <v>644</v>
       </c>
@@ -28429,7 +28424,7 @@
         <v>4.2857142857142856</v>
       </c>
     </row>
-    <row r="165" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A165" s="64" t="s">
         <v>645</v>
       </c>
@@ -28552,7 +28547,7 @@
         <v>0.89768559755339483</v>
       </c>
     </row>
-    <row r="166" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A166" s="64" t="s">
         <v>646</v>
       </c>
@@ -28675,7 +28670,7 @@
         <v>0.84488056240319498</v>
       </c>
     </row>
-    <row r="167" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A167" s="64" t="s">
         <v>647</v>
       </c>
@@ -28798,7 +28793,7 @@
         <v>0.79115858344502654</v>
       </c>
     </row>
-    <row r="168" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A168" s="64" t="s">
         <v>648</v>
       </c>
@@ -28921,7 +28916,7 @@
         <v>0.77406888933587614</v>
       </c>
     </row>
-    <row r="169" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A169" s="64" t="s">
         <v>649</v>
       </c>
@@ -29044,7 +29039,7 @@
         <v>0.95007407159306967</v>
       </c>
     </row>
-    <row r="170" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A170" s="64" t="s">
         <v>650</v>
       </c>
@@ -29167,7 +29162,7 @@
         <v>1.6504684110205614</v>
       </c>
     </row>
-    <row r="171" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A171" s="64" t="s">
         <v>650</v>
       </c>
@@ -29290,7 +29285,7 @@
         <v>1.5959766651655141</v>
       </c>
     </row>
-    <row r="172" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A172" s="64" t="s">
         <v>650</v>
       </c>
@@ -29413,7 +29408,7 @@
         <v>1.541459129098488</v>
       </c>
     </row>
-    <row r="173" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A173" s="64" t="s">
         <v>650</v>
       </c>
@@ -29536,7 +29531,7 @@
         <v>1.4870446603133847</v>
       </c>
     </row>
-    <row r="174" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A174" s="64" t="s">
         <v>651</v>
       </c>
@@ -29659,7 +29654,7 @@
         <v>1.29803634535601</v>
       </c>
     </row>
-    <row r="175" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A175" s="64" t="s">
         <v>652</v>
       </c>
@@ -29782,7 +29777,7 @@
         <v>1.2979593269679877</v>
       </c>
     </row>
-    <row r="176" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A176" s="64" t="s">
         <v>653</v>
       </c>
@@ -29905,7 +29900,7 @@
         <v>1.6263477020219728</v>
       </c>
     </row>
-    <row r="177" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A177" s="64" t="s">
         <v>654</v>
       </c>
@@ -30028,7 +30023,7 @@
         <v>1.2592386722239013</v>
       </c>
     </row>
-    <row r="178" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A178" s="64" t="s">
         <v>655</v>
       </c>
@@ -30151,7 +30146,7 @@
         <v>1.4641218723147973</v>
       </c>
     </row>
-    <row r="179" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A179" s="64" t="s">
         <v>656</v>
       </c>
@@ -30274,7 +30269,7 @@
         <v>1.6857797571068185</v>
       </c>
     </row>
-    <row r="180" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A180" s="64" t="s">
         <v>656</v>
       </c>
@@ -30397,7 +30392,7 @@
         <v>1.6461735009491525</v>
       </c>
     </row>
-    <row r="181" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A181" s="64" t="s">
         <v>657</v>
       </c>
@@ -30520,7 +30515,7 @@
         <v>1.5931435361112869</v>
       </c>
     </row>
-    <row r="182" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A182" s="64" t="s">
         <v>658</v>
       </c>
@@ -30643,7 +30638,7 @@
         <v>1.4757143571699876</v>
       </c>
     </row>
-    <row r="183" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A183" s="64" t="s">
         <v>658</v>
       </c>
@@ -30766,7 +30761,7 @@
         <v>1.4374300869105257</v>
       </c>
     </row>
-    <row r="184" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A184" s="64" t="s">
         <v>658</v>
       </c>
@@ -30889,7 +30884,7 @@
         <v>1.3985631033192503</v>
       </c>
     </row>
-    <row r="185" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A185" s="64" t="s">
         <v>659</v>
       </c>
@@ -31012,7 +31007,7 @@
         <v>1.3826456374022646</v>
       </c>
     </row>
-    <row r="186" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A186" s="64" t="s">
         <v>660</v>
       </c>
@@ -31135,7 +31130,7 @@
         <v>0.47357002940963111</v>
       </c>
     </row>
-    <row r="187" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A187" s="64" t="s">
         <v>661</v>
       </c>
@@ -31258,7 +31253,7 @@
         <v>1.2597354394053424</v>
       </c>
     </row>
-    <row r="188" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A188" s="64" t="s">
         <v>662</v>
       </c>
@@ -31381,7 +31376,7 @@
         <v>1.1675517449568096</v>
       </c>
     </row>
-    <row r="189" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A189" s="64" t="s">
         <v>663</v>
       </c>
@@ -31504,7 +31499,7 @@
         <v>1.3696411756979359</v>
       </c>
     </row>
-    <row r="190" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A190" s="64" t="s">
         <v>663</v>
       </c>
@@ -31627,7 +31622,7 @@
         <v>1.350214188462304</v>
       </c>
     </row>
-    <row r="191" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A191" s="64" t="s">
         <v>664</v>
       </c>
@@ -31750,7 +31745,7 @@
         <v>1.2329454023052526</v>
       </c>
     </row>
-    <row r="192" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A192" s="64" t="s">
         <v>664</v>
       </c>
@@ -31873,7 +31868,7 @@
         <v>1.1957801977735603</v>
       </c>
     </row>
-    <row r="193" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A193" s="64" t="s">
         <v>665</v>
       </c>
@@ -31996,7 +31991,7 @@
         <v>1.1035853568830785</v>
       </c>
     </row>
-    <row r="194" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A194" s="64" t="s">
         <v>665</v>
       </c>
@@ -32119,7 +32114,7 @@
         <v>1.0659650406849812</v>
       </c>
     </row>
-    <row r="195" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A195" s="64" t="s">
         <v>665</v>
       </c>
@@ -32242,7 +32237,7 @@
         <v>2.1875</v>
       </c>
     </row>
-    <row r="196" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A196" s="64" t="s">
         <v>665</v>
       </c>
@@ -32365,7 +32360,7 @@
         <v>2.1875</v>
       </c>
     </row>
-    <row r="197" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A197" s="64" t="s">
         <v>665</v>
       </c>
@@ -32488,7 +32483,7 @@
         <v>2.1875</v>
       </c>
     </row>
-    <row r="198" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A198" s="64" t="s">
         <v>665</v>
       </c>
@@ -32611,7 +32606,7 @@
         <v>2.1875</v>
       </c>
     </row>
-    <row r="199" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A199" s="64" t="s">
         <v>665</v>
       </c>
@@ -32734,7 +32729,7 @@
         <v>2.1875</v>
       </c>
     </row>
-    <row r="200" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A200" s="64" t="s">
         <v>665</v>
       </c>
@@ -32857,7 +32852,7 @@
         <v>2.1875</v>
       </c>
     </row>
-    <row r="201" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A201" s="64" t="s">
         <v>666</v>
       </c>
@@ -32979,7 +32974,7 @@
         <v>1.6566885721095854</v>
       </c>
     </row>
-    <row r="202" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A202" s="64" t="s">
         <v>666</v>
       </c>
@@ -33101,7 +33096,7 @@
         <v>1.6346161037144891</v>
       </c>
     </row>
-    <row r="203" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A203" s="64" t="s">
         <v>667</v>
       </c>
@@ -33223,7 +33218,7 @@
         <v>1.5890770411330262</v>
       </c>
     </row>
-    <row r="204" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A204" s="64" t="s">
         <v>668</v>
       </c>
@@ -33346,7 +33341,7 @@
         <v>1.6348488056211639</v>
       </c>
     </row>
-    <row r="205" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A205" s="64" t="s">
         <v>669</v>
       </c>
@@ -33469,7 +33464,7 @@
         <v>1.3994784856987472</v>
       </c>
     </row>
-    <row r="206" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A206" s="64" t="s">
         <v>669</v>
       </c>
@@ -33592,7 +33587,7 @@
         <v>1.3761547970799959</v>
       </c>
     </row>
-    <row r="207" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A207" s="64" t="s">
         <v>670</v>
       </c>
@@ -33715,7 +33710,7 @@
         <v>1.2739382867033264</v>
       </c>
     </row>
-    <row r="208" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A208" s="64" t="s">
         <v>670</v>
       </c>
@@ -33838,7 +33833,7 @@
         <v>1.2513432560545719</v>
       </c>
     </row>
-    <row r="209" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A209" s="64" t="s">
         <v>670</v>
       </c>
@@ -33961,7 +33956,7 @@
         <v>1.2287862611479596</v>
       </c>
     </row>
-    <row r="210" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A210" s="64" t="s">
         <v>670</v>
       </c>
@@ -34084,7 +34079,7 @@
         <v>1.1838391039622553</v>
       </c>
     </row>
-    <row r="211" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A211" s="64" t="s">
         <v>671</v>
       </c>
@@ -34207,7 +34202,7 @@
         <v>1.3995973831143944</v>
       </c>
     </row>
-    <row r="212" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A212" s="64" t="s">
         <v>671</v>
       </c>
@@ -34330,7 +34325,7 @@
         <v>1.4269474786562346</v>
       </c>
     </row>
-    <row r="213" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A213" s="64" t="s">
         <v>672</v>
       </c>
@@ -34453,7 +34448,7 @@
         <v>1.4544075393871425</v>
       </c>
     </row>
-    <row r="214" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A214" s="64" t="s">
         <v>673</v>
       </c>
@@ -34576,7 +34571,7 @@
         <v>1.1915152802141717</v>
       </c>
     </row>
-    <row r="215" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A215" s="64" t="s">
         <v>674</v>
       </c>
@@ -34698,7 +34693,7 @@
         <v>1.3027775635825822</v>
       </c>
     </row>
-    <row r="216" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A216" s="64" t="s">
         <v>675</v>
       </c>
@@ -34820,7 +34815,7 @@
         <v>0.81407876134588997</v>
       </c>
     </row>
-    <row r="217" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A217" s="64" t="s">
         <v>676</v>
       </c>
@@ -34942,7 +34937,7 @@
         <v>1.1216996276148128</v>
       </c>
     </row>
-    <row r="218" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A218" s="64" t="s">
         <v>677</v>
       </c>
@@ -35065,7 +35060,7 @@
         <v>1.1919024331549293</v>
       </c>
     </row>
-    <row r="219" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A219" s="64" t="s">
         <v>678</v>
       </c>
@@ -35190,7 +35185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A220" s="64" t="s">
         <v>569</v>
       </c>
@@ -35315,7 +35310,7 @@
         <v>1.4778743985473446</v>
       </c>
     </row>
-    <row r="221" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A221" s="64" t="s">
         <v>569</v>
       </c>
@@ -35440,7 +35435,7 @@
         <v>1.4352282729652679</v>
       </c>
     </row>
-    <row r="222" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A222" s="64" t="s">
         <v>679</v>
       </c>
@@ -35557,7 +35552,7 @@
         <v>2.6923076923076925</v>
       </c>
     </row>
-    <row r="223" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A223" s="64" t="s">
         <v>680</v>
       </c>
@@ -35674,7 +35669,7 @@
         <v>3.378378378378379</v>
       </c>
     </row>
-    <row r="224" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A224" s="64" t="s">
         <v>680</v>
       </c>
@@ -35791,7 +35786,7 @@
         <v>3.378378378378379</v>
       </c>
     </row>
-    <row r="225" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A225" s="64" t="s">
         <v>680</v>
       </c>
@@ -35908,7 +35903,7 @@
         <v>3.3783783783783781</v>
       </c>
     </row>
-    <row r="226" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A226" s="64" t="s">
         <v>680</v>
       </c>
@@ -36025,7 +36020,7 @@
         <v>3.3783783783783781</v>
       </c>
     </row>
-    <row r="227" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A227" s="64" t="s">
         <v>680</v>
       </c>
@@ -36142,7 +36137,7 @@
         <v>3.3783783783783781</v>
       </c>
     </row>
-    <row r="228" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A228" s="64" t="s">
         <v>680</v>
       </c>
@@ -36259,7 +36254,7 @@
         <v>3.3783783783783785</v>
       </c>
     </row>
-    <row r="229" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A229" s="64" t="s">
         <v>680</v>
       </c>
@@ -36376,7 +36371,7 @@
         <v>3.3783783783783781</v>
       </c>
     </row>
-    <row r="230" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A230" s="64" t="s">
         <v>680</v>
       </c>
@@ -36493,7 +36488,7 @@
         <v>3.3783783783783785</v>
       </c>
     </row>
-    <row r="231" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A231" s="83" t="s">
         <v>720</v>
       </c>
@@ -36517,7 +36512,9 @@
         <v>196</v>
       </c>
       <c r="M231" s="74"/>
-      <c r="N231" s="65"/>
+      <c r="N231" s="65" t="s">
+        <v>26</v>
+      </c>
       <c r="O231" s="67" t="s">
         <v>712</v>
       </c>
@@ -36598,7 +36595,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="232" spans="1:42" s="95" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:42" s="95" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A232" s="89" t="s">
         <v>721</v>
       </c>
@@ -36622,7 +36619,9 @@
         <v>212</v>
       </c>
       <c r="M232" s="74"/>
-      <c r="N232" s="67"/>
+      <c r="N232" s="65" t="s">
+        <v>26</v>
+      </c>
       <c r="O232" s="67" t="s">
         <v>711</v>
       </c>
@@ -36699,7 +36698,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="233" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A233" s="64" t="s">
         <v>729</v>
       </c>
@@ -36723,7 +36722,7 @@
         <v>221</v>
       </c>
       <c r="M233" s="74"/>
-      <c r="N233" s="6" t="s">
+      <c r="N233" s="65" t="s">
         <v>26</v>
       </c>
       <c r="O233" s="5" t="s">
@@ -36802,7 +36801,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="234" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A234" s="83" t="s">
         <v>722</v>
       </c>
@@ -36904,7 +36903,7 @@
         <v>2.2839969947407965</v>
       </c>
     </row>
-    <row r="235" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A235" s="83" t="s">
         <v>723</v>
       </c>
@@ -37004,7 +37003,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="236" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A236" s="83" t="s">
         <v>724</v>
       </c>
@@ -37104,7 +37103,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="237" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A237" s="83" t="s">
         <v>725</v>
       </c>
@@ -37204,7 +37203,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="238" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A238" s="83" t="s">
         <v>726</v>
       </c>
@@ -37227,7 +37226,9 @@
         <v>708</v>
       </c>
       <c r="M238" s="99"/>
-      <c r="N238" s="65"/>
+      <c r="N238" s="65" t="s">
+        <v>26</v>
+      </c>
       <c r="O238" s="67" t="s">
         <v>712</v>
       </c>
@@ -37304,7 +37305,7 @@
         <v>3.2456799398948157</v>
       </c>
     </row>
-    <row r="239" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A239" s="83" t="s">
         <v>727</v>
       </c>
@@ -37404,7 +37405,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="240" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A240" s="83" t="s">
         <v>728</v>
       </c>
@@ -37504,7 +37505,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="241" spans="1:42" s="64" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:42" s="64" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A241" s="64" t="s">
         <v>733</v>
       </c>
@@ -37526,20 +37527,20 @@
         <v>732</v>
       </c>
       <c r="M241" s="110"/>
-      <c r="N241" s="111" t="s">
+      <c r="N241" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="O241" s="112"/>
-      <c r="P241" s="113" t="s">
+      <c r="O241" s="111"/>
+      <c r="P241" s="112" t="s">
         <v>27</v>
       </c>
       <c r="R241" s="103">
         <v>0.72499999999999998</v>
       </c>
-      <c r="S241" s="114">
+      <c r="S241" s="113">
         <v>0.27500000000000002</v>
       </c>
-      <c r="T241" s="115">
+      <c r="T241" s="114">
         <f t="shared" si="39"/>
         <v>1</v>
       </c>
@@ -37553,7 +37554,7 @@
       <c r="AB241" s="78">
         <v>1669.242</v>
       </c>
-      <c r="AC241" s="116"/>
+      <c r="AC241" s="115"/>
       <c r="AD241" s="68"/>
       <c r="AE241" s="68"/>
       <c r="AF241" s="68"/>
@@ -37873,9 +37874,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AA5B41D-754B-41F4-AE3E-2CEADDCF305E}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>568</v>
       </c>

</xml_diff>

<commit_message>
alterado xlxs e gerar_data.py
</commit_message>
<xml_diff>
--- a/areas_land_bank_com_id.xlsx
+++ b/areas_land_bank_com_id.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinicius.castro\Documents\01 Profissional\Buriti Empreendimentos\Repositórios\land-bank-mapa-brasil-terrenos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5256DE6A-6317-4F17-9C7A-ABDC3532BCF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C596D42-BED9-49AD-8EFE-00C9C890A74F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2D7381EB-1656-47BB-A82F-14AB3B13CCCD}"/>
   </bookViews>
@@ -5306,7 +5306,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2195" uniqueCount="737">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2195" uniqueCount="738">
   <si>
     <t>Nome</t>
   </si>
@@ -7522,6 +7522,9 @@
   </si>
   <si>
     <t>CENTRO-OESTE</t>
+  </si>
+  <si>
+    <t>a DEFINIR</t>
   </si>
 </sst>
 </file>
@@ -7870,7 +7873,7 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -8158,6 +8161,7 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -8551,7 +8555,8 @@
     <col min="32" max="32" width="12.21875" customWidth="1"/>
     <col min="33" max="33" width="8.77734375" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.5546875" customWidth="1"/>
+    <col min="35" max="35" width="10.77734375" customWidth="1"/>
+    <col min="36" max="36" width="9.5546875" customWidth="1"/>
     <col min="37" max="38" width="9" customWidth="1"/>
     <col min="39" max="39" width="16" bestFit="1" customWidth="1"/>
     <col min="40" max="41" width="12.77734375" customWidth="1"/>
@@ -36512,8 +36517,8 @@
         <v>196</v>
       </c>
       <c r="M231" s="74"/>
-      <c r="N231" s="65" t="s">
-        <v>26</v>
+      <c r="N231" s="101" t="s">
+        <v>737</v>
       </c>
       <c r="O231" s="67" t="s">
         <v>712</v>
@@ -36619,8 +36624,8 @@
         <v>212</v>
       </c>
       <c r="M232" s="74"/>
-      <c r="N232" s="65" t="s">
-        <v>26</v>
+      <c r="N232" s="101" t="s">
+        <v>737</v>
       </c>
       <c r="O232" s="67" t="s">
         <v>711</v>
@@ -36722,7 +36727,7 @@
         <v>221</v>
       </c>
       <c r="M233" s="74"/>
-      <c r="N233" s="65" t="s">
+      <c r="N233" s="6" t="s">
         <v>26</v>
       </c>
       <c r="O233" s="5" t="s">
@@ -37226,8 +37231,8 @@
         <v>708</v>
       </c>
       <c r="M238" s="99"/>
-      <c r="N238" s="65" t="s">
-        <v>26</v>
+      <c r="N238" s="101" t="s">
+        <v>737</v>
       </c>
       <c r="O238" s="67" t="s">
         <v>712</v>
@@ -37527,20 +37532,20 @@
         <v>732</v>
       </c>
       <c r="M241" s="110"/>
-      <c r="N241" s="65" t="s">
+      <c r="N241" s="111" t="s">
         <v>26</v>
       </c>
-      <c r="O241" s="111"/>
-      <c r="P241" s="112" t="s">
+      <c r="O241" s="112"/>
+      <c r="P241" s="113" t="s">
         <v>27</v>
       </c>
       <c r="R241" s="103">
         <v>0.72499999999999998</v>
       </c>
-      <c r="S241" s="113">
+      <c r="S241" s="114">
         <v>0.27500000000000002</v>
       </c>
-      <c r="T241" s="114">
+      <c r="T241" s="115">
         <f t="shared" si="39"/>
         <v>1</v>
       </c>
@@ -37554,7 +37559,7 @@
       <c r="AB241" s="78">
         <v>1669.242</v>
       </c>
-      <c r="AC241" s="115"/>
+      <c r="AC241" s="116"/>
       <c r="AD241" s="68"/>
       <c r="AE241" s="68"/>
       <c r="AF241" s="68"/>

</xml_diff>

<commit_message>
adicionando dados MAP 135 e 136
</commit_message>
<xml_diff>
--- a/areas_land_bank_com_id.xlsx
+++ b/areas_land_bank_com_id.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Departamento Controladoria\3 - BT 360º\Landbank\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{527FC402-853E-414E-9886-EC808F900A5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{058A33A0-DEE3-47FE-8F5A-E5A2CA5ABC9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="960" windowWidth="29040" windowHeight="15720" xr2:uid="{2D7381EB-1656-47BB-A82F-14AB3B13CCCD}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Planilha2" sheetId="3" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">AREAS!$A$1:$AK$242</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">AREAS!$A$1:$AK$244</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -5328,7 +5328,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2389" uniqueCount="786">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2651" uniqueCount="795">
   <si>
     <t>Nome</t>
   </si>
@@ -7704,6 +7704,33 @@
   </si>
   <si>
     <t>MAP134</t>
+  </si>
+  <si>
+    <t>MUNARO EMPREENDIMENTOS IMOBILIÁRIOS LTDA</t>
+  </si>
+  <si>
+    <t>Status da área</t>
+  </si>
+  <si>
+    <t>Estudo de viabilidade</t>
+  </si>
+  <si>
+    <t>LandBank</t>
+  </si>
+  <si>
+    <t>GUARANTÃ DO NORTE</t>
+  </si>
+  <si>
+    <t>PERGENTINO DE VASCONCELOS JUNIOR</t>
+  </si>
+  <si>
+    <t>SEDESTE</t>
+  </si>
+  <si>
+    <t>MAP135</t>
+  </si>
+  <si>
+    <t>MAP136</t>
   </si>
 </sst>
 </file>
@@ -7831,7 +7858,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -7877,12 +7904,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -7969,7 +7990,7 @@
     <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -8056,7 +8077,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="37" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="37" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -8072,7 +8093,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -8080,9 +8101,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -8105,26 +8126,25 @@
     <xf numFmtId="49" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="37" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="37" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -8136,7 +8156,23 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -8491,7 +8527,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BB1E7F9-B7E0-4EE5-A96E-08F27078CA81}">
   <sheetPr codeName="Folha1"/>
-  <dimension ref="A1:AN242"/>
+  <dimension ref="A1:AO244"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.1796875" customWidth="1"/>
@@ -8508,7 +8544,7 @@
     <col min="13" max="13" width="53.36328125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="19.453125" style="3" customWidth="1"/>
     <col min="15" max="15" width="14.54296875" customWidth="1"/>
-    <col min="16" max="16" width="9.1796875" customWidth="1"/>
+    <col min="16" max="16" width="9.1796875" style="3" customWidth="1"/>
     <col min="17" max="17" width="10" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12.81640625" customWidth="1"/>
     <col min="19" max="19" width="11.54296875" customWidth="1"/>
@@ -8531,9 +8567,10 @@
     <col min="37" max="37" width="17.453125" bestFit="1" customWidth="1"/>
     <col min="38" max="39" width="12.81640625" customWidth="1"/>
     <col min="40" max="40" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="23.08984375" style="76" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" ht="50" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:41" ht="50" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>432</v>
       </c>
@@ -8654,8 +8691,11 @@
       <c r="AN1" s="9" t="s">
         <v>550</v>
       </c>
+      <c r="AO1" s="74" t="s">
+        <v>787</v>
+      </c>
     </row>
-    <row r="2" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>440</v>
       </c>
@@ -8769,8 +8809,11 @@
         <f>AI2*AM2/(AD2+AB2)</f>
         <v>3.3809797786673061</v>
       </c>
+      <c r="AO2" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="3" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>441</v>
       </c>
@@ -8864,7 +8907,7 @@
         <v>384.77817538189237</v>
       </c>
       <c r="AI3" s="21">
-        <f t="shared" ref="AI2:AI65" si="6">(AH3*AG3*AF3)/10^6</f>
+        <f t="shared" ref="AI3:AI65" si="6">(AH3*AG3*AF3)/10^6</f>
         <v>4.3</v>
       </c>
       <c r="AJ3" s="21">
@@ -8886,8 +8929,11 @@
         <f t="shared" ref="AN3:AN66" si="8">AI3*AM3/(AD3+AB3)</f>
         <v>4.8097271922736544</v>
       </c>
+      <c r="AO3" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="4" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>441</v>
       </c>
@@ -9003,8 +9049,11 @@
         <f t="shared" si="8"/>
         <v>5.3580126643935699</v>
       </c>
+      <c r="AO4" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="5" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>493</v>
       </c>
@@ -9124,8 +9173,11 @@
         <f t="shared" si="8"/>
         <v>1.1478379123898736</v>
       </c>
+      <c r="AO5" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="6" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>481</v>
       </c>
@@ -9245,8 +9297,11 @@
         <f t="shared" si="8"/>
         <v>0.90690345120653837</v>
       </c>
+      <c r="AO6" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="7" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>482</v>
       </c>
@@ -9366,8 +9421,11 @@
         <f t="shared" si="8"/>
         <v>0.87259450365707092</v>
       </c>
+      <c r="AO7" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="8" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>483</v>
       </c>
@@ -9487,8 +9545,11 @@
         <f t="shared" si="8"/>
         <v>0.83860953776262182</v>
       </c>
+      <c r="AO8" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="9" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>483</v>
       </c>
@@ -9608,8 +9669,11 @@
         <f t="shared" si="8"/>
         <v>0.80502313984963059</v>
       </c>
+      <c r="AO9" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="10" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>483</v>
       </c>
@@ -9729,8 +9793,11 @@
         <f t="shared" si="8"/>
         <v>2.024472392638037</v>
       </c>
+      <c r="AO10" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="11" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>434</v>
       </c>
@@ -9841,11 +9908,14 @@
         <v>1</v>
       </c>
       <c r="AN11" s="51" t="e">
-        <f t="shared" si="8"/>
+        <f>AI11*AM11/(AD11+AB11)</f>
         <v>#DIV/0!</v>
       </c>
+      <c r="AO11" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="12" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>435</v>
       </c>
@@ -9959,8 +10029,11 @@
         <f t="shared" si="8"/>
         <v>3.2306536438767841</v>
       </c>
+      <c r="AO12" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="13" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>436</v>
       </c>
@@ -10074,8 +10147,11 @@
         <f t="shared" si="8"/>
         <v>4.883546205860255</v>
       </c>
+      <c r="AO13" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="14" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>436</v>
       </c>
@@ -10189,8 +10265,11 @@
         <f t="shared" si="8"/>
         <v>4.883546205860255</v>
       </c>
+      <c r="AO14" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="15" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>437</v>
       </c>
@@ -10304,8 +10383,11 @@
         <f t="shared" si="8"/>
         <v>3.7565740045078888</v>
       </c>
+      <c r="AO15" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="16" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>438</v>
       </c>
@@ -10419,8 +10501,11 @@
         <f t="shared" si="8"/>
         <v>3.7565740045078897</v>
       </c>
+      <c r="AO16" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="17" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>439</v>
       </c>
@@ -10534,8 +10619,11 @@
         <f t="shared" si="8"/>
         <v>3.7565740045078893</v>
       </c>
+      <c r="AO17" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="18" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>444</v>
       </c>
@@ -10649,8 +10737,11 @@
         <f t="shared" si="8"/>
         <v>3.230653643876785</v>
       </c>
+      <c r="AO18" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="19" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>445</v>
       </c>
@@ -10764,8 +10855,11 @@
         <f t="shared" si="8"/>
         <v>2.9301277235161534</v>
       </c>
+      <c r="AO19" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="20" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>445</v>
       </c>
@@ -10879,8 +10973,11 @@
         <f t="shared" si="8"/>
         <v>2.9301277235161534</v>
       </c>
+      <c r="AO20" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="21" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>445</v>
       </c>
@@ -10994,8 +11091,11 @@
         <f t="shared" si="8"/>
         <v>2.9301277235161534</v>
       </c>
+      <c r="AO21" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="22" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>445</v>
       </c>
@@ -11109,8 +11209,11 @@
         <f t="shared" si="8"/>
         <v>2.9301277235161534</v>
       </c>
+      <c r="AO22" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="23" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>445</v>
       </c>
@@ -11224,8 +11327,11 @@
         <f t="shared" si="8"/>
         <v>2.9301277235161534</v>
       </c>
+      <c r="AO23" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="24" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>445</v>
       </c>
@@ -11339,8 +11445,11 @@
         <f t="shared" si="8"/>
         <v>2.9301277235161534</v>
       </c>
+      <c r="AO24" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="25" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>445</v>
       </c>
@@ -11454,8 +11563,11 @@
         <f t="shared" si="8"/>
         <v>2.9301277235161534</v>
       </c>
+      <c r="AO25" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="26" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>446</v>
       </c>
@@ -11569,8 +11681,11 @@
         <f t="shared" si="8"/>
         <v>0.83115017886351839</v>
       </c>
+      <c r="AO26" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="27" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>447</v>
       </c>
@@ -11684,8 +11799,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO27" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="28" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>447</v>
       </c>
@@ -11798,8 +11916,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO28" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="29" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>447</v>
       </c>
@@ -11913,8 +12034,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO29" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="30" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>447</v>
       </c>
@@ -12028,8 +12152,11 @@
         <f t="shared" si="8"/>
         <v>4.140625</v>
       </c>
+      <c r="AO30" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="31" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>447</v>
       </c>
@@ -12143,8 +12270,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO31" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="32" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
         <v>447</v>
       </c>
@@ -12258,8 +12388,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO32" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="33" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>447</v>
       </c>
@@ -12373,8 +12506,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO33" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="34" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>447</v>
       </c>
@@ -12488,8 +12624,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO34" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="35" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>447</v>
       </c>
@@ -12603,8 +12742,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO35" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="36" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>447</v>
       </c>
@@ -12718,8 +12860,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO36" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="37" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
         <v>447</v>
       </c>
@@ -12833,8 +12978,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO37" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="38" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
         <v>447</v>
       </c>
@@ -12948,8 +13096,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO38" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="39" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>447</v>
       </c>
@@ -13063,8 +13214,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO39" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="40" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
         <v>447</v>
       </c>
@@ -13178,8 +13332,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO40" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="41" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>447</v>
       </c>
@@ -13293,8 +13450,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO41" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="42" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>447</v>
       </c>
@@ -13408,8 +13568,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO42" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="43" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>447</v>
       </c>
@@ -13523,8 +13686,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO43" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="44" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>447</v>
       </c>
@@ -13638,8 +13804,11 @@
         <f t="shared" si="8"/>
         <v>4.296875</v>
       </c>
+      <c r="AO44" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="45" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>447</v>
       </c>
@@ -13753,8 +13922,11 @@
         <f t="shared" si="8"/>
         <v>3.90625</v>
       </c>
+      <c r="AO45" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="46" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>448</v>
       </c>
@@ -13874,8 +14046,11 @@
         <f t="shared" si="8"/>
         <v>1.5033333068541384</v>
       </c>
+      <c r="AO46" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="47" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>448</v>
       </c>
@@ -13995,8 +14170,11 @@
         <f t="shared" si="8"/>
         <v>1.5033333068541381</v>
       </c>
+      <c r="AO47" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="48" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>448</v>
       </c>
@@ -14116,8 +14294,11 @@
         <f t="shared" si="8"/>
         <v>1.1881369949110563</v>
       </c>
+      <c r="AO48" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="49" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>448</v>
       </c>
@@ -14237,8 +14418,11 @@
         <f t="shared" si="8"/>
         <v>1.1629101414416052</v>
       </c>
+      <c r="AO49" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="50" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
         <v>449</v>
       </c>
@@ -14351,8 +14535,11 @@
         <f t="shared" si="8"/>
         <v>3.9062500000000004</v>
       </c>
+      <c r="AO50" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="51" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
         <v>451</v>
       </c>
@@ -14466,8 +14653,11 @@
         <f t="shared" si="8"/>
         <v>4.6875000000000009</v>
       </c>
+      <c r="AO51" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="52" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
         <v>483</v>
       </c>
@@ -14587,8 +14777,11 @@
         <f t="shared" si="8"/>
         <v>2.024472392638037</v>
       </c>
+      <c r="AO52" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="53" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
         <v>483</v>
       </c>
@@ -14708,8 +14901,11 @@
         <f t="shared" si="8"/>
         <v>2.024472392638037</v>
       </c>
+      <c r="AO53" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="54" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
         <v>483</v>
       </c>
@@ -14829,8 +15025,11 @@
         <f t="shared" si="8"/>
         <v>2.024472392638037</v>
       </c>
+      <c r="AO54" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="55" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
         <v>483</v>
       </c>
@@ -14950,8 +15149,11 @@
         <f t="shared" si="8"/>
         <v>2.024472392638037</v>
       </c>
+      <c r="AO55" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="56" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
         <v>455</v>
       </c>
@@ -15071,8 +15273,11 @@
         <f t="shared" si="8"/>
         <v>2.0794444816235882</v>
       </c>
+      <c r="AO56" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="57" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
         <v>455</v>
       </c>
@@ -15191,8 +15396,11 @@
         <f t="shared" si="8"/>
         <v>0.682062825375507</v>
       </c>
+      <c r="AO57" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="58" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A58" s="6" t="s">
         <v>454</v>
       </c>
@@ -15312,8 +15520,11 @@
         <f t="shared" si="8"/>
         <v>1.584067227618178</v>
       </c>
+      <c r="AO58" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="59" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
         <v>456</v>
       </c>
@@ -15433,8 +15644,11 @@
         <f t="shared" si="8"/>
         <v>1.2626874796242238</v>
       </c>
+      <c r="AO59" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="60" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A60" s="6" t="s">
         <v>457</v>
       </c>
@@ -15554,8 +15768,11 @@
         <f t="shared" si="8"/>
         <v>1.165542478997921</v>
       </c>
+      <c r="AO60" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="61" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
         <v>457</v>
       </c>
@@ -15675,8 +15892,11 @@
         <f t="shared" si="8"/>
         <v>1.1453025708336924</v>
       </c>
+      <c r="AO61" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="62" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A62" s="6" t="s">
         <v>458</v>
       </c>
@@ -15796,8 +16016,11 @@
         <f t="shared" si="8"/>
         <v>1.0499523822058021</v>
       </c>
+      <c r="AO62" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="63" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A63" s="6" t="s">
         <v>459</v>
       </c>
@@ -15911,8 +16134,11 @@
         <f t="shared" si="8"/>
         <v>3.9384920139218527</v>
       </c>
+      <c r="AO63" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="64" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
         <v>459</v>
       </c>
@@ -16026,8 +16252,11 @@
         <f t="shared" si="8"/>
         <v>3.9384920139218527</v>
       </c>
+      <c r="AO64" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="65" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>459</v>
       </c>
@@ -16141,8 +16370,11 @@
         <f t="shared" si="8"/>
         <v>3.9384920139218527</v>
       </c>
+      <c r="AO65" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="66" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
         <v>460</v>
       </c>
@@ -16256,8 +16488,11 @@
         <f t="shared" si="8"/>
         <v>3.5833333333333335</v>
       </c>
+      <c r="AO66" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="67" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
         <v>461</v>
       </c>
@@ -16371,8 +16606,11 @@
         <f t="shared" ref="AN67:AN130" si="19">AI67*AM67/(AD67+AB67)</f>
         <v>3.8333333333333335</v>
       </c>
+      <c r="AO67" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="68" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A68" s="6" t="s">
         <v>462</v>
       </c>
@@ -16486,8 +16724,11 @@
         <f t="shared" si="19"/>
         <v>3.5833333333333335</v>
       </c>
+      <c r="AO68" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="69" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
         <v>462</v>
       </c>
@@ -16601,8 +16842,11 @@
         <f t="shared" si="19"/>
         <v>3.5833333333333335</v>
       </c>
+      <c r="AO69" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="70" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
         <v>463</v>
       </c>
@@ -16721,8 +16965,11 @@
         <f t="shared" si="19"/>
         <v>1.6840907460634127</v>
       </c>
+      <c r="AO70" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="71" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
         <v>464</v>
       </c>
@@ -16841,8 +17088,11 @@
         <f t="shared" si="19"/>
         <v>1.7104564330775569</v>
       </c>
+      <c r="AO71" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="72" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A72" s="6" t="s">
         <v>464</v>
       </c>
@@ -16961,8 +17211,11 @@
         <f t="shared" si="19"/>
         <v>1.6579735962048303</v>
       </c>
+      <c r="AO72" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="73" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A73" s="6" t="s">
         <v>465</v>
       </c>
@@ -17081,8 +17334,11 @@
         <f t="shared" si="19"/>
         <v>2.5287610566591523</v>
       </c>
+      <c r="AO73" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="74" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
         <v>465</v>
       </c>
@@ -17201,8 +17457,11 @@
         <f t="shared" si="19"/>
         <v>2.4793535855822042</v>
       </c>
+      <c r="AO74" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="75" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
         <v>466</v>
       </c>
@@ -17324,8 +17583,11 @@
         <f t="shared" si="19"/>
         <v>1.890388055872956</v>
       </c>
+      <c r="AO75" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="76" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A76" s="6" t="s">
         <v>466</v>
       </c>
@@ -17447,8 +17709,11 @@
         <f t="shared" si="19"/>
         <v>1.8605083275965164</v>
       </c>
+      <c r="AO76" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="77" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
         <v>467</v>
       </c>
@@ -17570,8 +17835,11 @@
         <f t="shared" si="19"/>
         <v>1.8523399895648596</v>
       </c>
+      <c r="AO77" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="78" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A78" s="6" t="s">
         <v>467</v>
       </c>
@@ -17693,8 +17961,11 @@
         <f t="shared" si="19"/>
         <v>1.7669888872138106</v>
       </c>
+      <c r="AO78" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="79" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
         <v>468</v>
       </c>
@@ -17814,8 +18085,11 @@
         <f t="shared" si="19"/>
         <v>0.64100515446669049</v>
       </c>
+      <c r="AO79" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="80" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
         <v>468</v>
       </c>
@@ -17935,8 +18209,11 @@
         <f t="shared" si="19"/>
         <v>0.62670976763932151</v>
       </c>
+      <c r="AO80" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="81" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A81" s="6" t="s">
         <v>469</v>
       </c>
@@ -18056,8 +18333,11 @@
         <f t="shared" si="19"/>
         <v>0.76883870310314895</v>
       </c>
+      <c r="AO81" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="82" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
         <v>475</v>
       </c>
@@ -18177,8 +18457,11 @@
         <f t="shared" si="19"/>
         <v>1.2072988815514583</v>
       </c>
+      <c r="AO82" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="83" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A83" s="6" t="s">
         <v>471</v>
       </c>
@@ -18298,8 +18581,11 @@
         <f t="shared" si="19"/>
         <v>0.83525452781953513</v>
       </c>
+      <c r="AO83" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="84" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
         <v>471</v>
       </c>
@@ -18419,8 +18705,11 @@
         <f t="shared" si="19"/>
         <v>0.81799598953212038</v>
       </c>
+      <c r="AO84" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="85" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A85" s="6" t="s">
         <v>471</v>
       </c>
@@ -18540,8 +18829,11 @@
         <f t="shared" si="19"/>
         <v>0.78388138912123639</v>
       </c>
+      <c r="AO85" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="86" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
         <v>472</v>
       </c>
@@ -18661,8 +18953,11 @@
         <f t="shared" si="19"/>
         <v>1.1501266268686077</v>
       </c>
+      <c r="AO86" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="87" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A87" s="6" t="s">
         <v>473</v>
       </c>
@@ -18782,8 +19077,11 @@
         <f t="shared" si="19"/>
         <v>0.23299756298435631</v>
       </c>
+      <c r="AO87" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="88" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A88" s="6" t="s">
         <v>473</v>
       </c>
@@ -18903,8 +19201,11 @@
         <f t="shared" si="19"/>
         <v>1.2387943662501089</v>
       </c>
+      <c r="AO88" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="89" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
         <v>474</v>
       </c>
@@ -19024,8 +19325,11 @@
         <f t="shared" si="19"/>
         <v>1.5149909654595908</v>
       </c>
+      <c r="AO89" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="90" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A90" s="6" t="s">
         <v>546</v>
       </c>
@@ -19145,8 +19449,11 @@
         <f t="shared" si="19"/>
         <v>1.2046020634661616</v>
       </c>
+      <c r="AO90" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="91" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A91" s="6" t="s">
         <v>475</v>
       </c>
@@ -19266,8 +19573,11 @@
         <f t="shared" si="19"/>
         <v>1.4090811331942312</v>
       </c>
+      <c r="AO91" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="92" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A92" s="6" t="s">
         <v>475</v>
       </c>
@@ -19387,8 +19697,11 @@
         <f t="shared" si="19"/>
         <v>1.1397336017719824</v>
       </c>
+      <c r="AO92" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="93" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A93" s="6" t="s">
         <v>475</v>
       </c>
@@ -19508,8 +19821,11 @@
         <f t="shared" si="19"/>
         <v>1.0959959051299162</v>
       </c>
+      <c r="AO93" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="94" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
         <v>475</v>
       </c>
@@ -19629,8 +19945,11 @@
         <f t="shared" si="19"/>
         <v>1.0527200029561115</v>
       </c>
+      <c r="AO94" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="95" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A95" s="6" t="s">
         <v>545</v>
       </c>
@@ -19744,8 +20063,11 @@
         <f t="shared" si="19"/>
         <v>3.2407407407407409</v>
       </c>
+      <c r="AO95" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="96" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A96" s="6" t="s">
         <v>476</v>
       </c>
@@ -19865,8 +20187,11 @@
         <f t="shared" si="19"/>
         <v>2.1202973983797322</v>
       </c>
+      <c r="AO96" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="97" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A97" s="6" t="s">
         <v>477</v>
       </c>
@@ -19986,8 +20311,11 @@
         <f t="shared" si="19"/>
         <v>2.0772596632135061</v>
       </c>
+      <c r="AO97" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="98" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A98" s="6" t="s">
         <v>450</v>
       </c>
@@ -20101,8 +20429,11 @@
         <f t="shared" si="19"/>
         <v>3.2407407407407409</v>
       </c>
+      <c r="AO98" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="99" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A99" s="6" t="s">
         <v>452</v>
       </c>
@@ -20216,8 +20547,11 @@
         <f t="shared" si="19"/>
         <v>6.2499999999999991</v>
       </c>
+      <c r="AO99" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="100" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A100" s="6" t="s">
         <v>479</v>
       </c>
@@ -20337,8 +20671,11 @@
         <f t="shared" si="19"/>
         <v>1.5361651825388483</v>
       </c>
+      <c r="AO100" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="101" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A101" s="6" t="s">
         <v>479</v>
       </c>
@@ -20458,8 +20795,11 @@
         <f t="shared" si="19"/>
         <v>1.5065784699927574</v>
       </c>
+      <c r="AO101" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="102" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A102" s="6" t="s">
         <v>479</v>
       </c>
@@ -20579,8 +20919,11 @@
         <f t="shared" si="19"/>
         <v>1.4478450040383797</v>
       </c>
+      <c r="AO102" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="103" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A103" s="6" t="s">
         <v>480</v>
       </c>
@@ -20700,8 +21043,11 @@
         <f t="shared" si="19"/>
         <v>1.6691380981214541</v>
       </c>
+      <c r="AO103" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="104" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A104" s="6" t="s">
         <v>480</v>
       </c>
@@ -20821,8 +21167,11 @@
         <f t="shared" si="19"/>
         <v>1.6065963825333243</v>
       </c>
+      <c r="AO104" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="105" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A105" s="6" t="s">
         <v>478</v>
       </c>
@@ -20942,8 +21291,11 @@
         <f t="shared" si="19"/>
         <v>1.0994472988394468</v>
       </c>
+      <c r="AO105" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="106" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A106" s="6" t="s">
         <v>478</v>
       </c>
@@ -21063,8 +21415,11 @@
         <f t="shared" si="19"/>
         <v>1.0586916755795146</v>
       </c>
+      <c r="AO106" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="107" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A107" s="6" t="s">
         <v>442</v>
       </c>
@@ -21178,8 +21533,11 @@
         <f t="shared" si="19"/>
         <v>4.5078888054094666</v>
       </c>
+      <c r="AO107" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="108" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A108" s="6" t="s">
         <v>443</v>
       </c>
@@ -21293,8 +21651,11 @@
         <f t="shared" si="19"/>
         <v>4.5078888054094675</v>
       </c>
+      <c r="AO108" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="109" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A109" s="6" t="s">
         <v>443</v>
       </c>
@@ -21408,8 +21769,11 @@
         <f t="shared" si="19"/>
         <v>4.5078888054094666</v>
       </c>
+      <c r="AO109" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="110" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A110" s="6" t="s">
         <v>443</v>
       </c>
@@ -21523,8 +21887,11 @@
         <f t="shared" si="19"/>
         <v>4.5078888054094683</v>
       </c>
+      <c r="AO110" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="111" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A111" s="6" t="s">
         <v>443</v>
       </c>
@@ -21638,8 +22005,11 @@
         <f t="shared" si="19"/>
         <v>4.5078888054094683</v>
       </c>
+      <c r="AO111" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="112" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A112" s="6" t="s">
         <v>443</v>
       </c>
@@ -21753,8 +22123,11 @@
         <f t="shared" si="19"/>
         <v>4.5078888054094683</v>
       </c>
+      <c r="AO112" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="113" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A113" s="6" t="s">
         <v>453</v>
       </c>
@@ -21867,8 +22240,11 @@
         <f t="shared" si="19"/>
         <v>3.7037037037037033</v>
       </c>
+      <c r="AO113" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="114" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A114" s="6" t="s">
         <v>484</v>
       </c>
@@ -21988,8 +22364,11 @@
         <f t="shared" si="19"/>
         <v>0.73245167478536033</v>
       </c>
+      <c r="AO114" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="115" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A115" s="6" t="s">
         <v>485</v>
       </c>
@@ -22109,8 +22488,11 @@
         <f t="shared" si="19"/>
         <v>0.70127185350915722</v>
       </c>
+      <c r="AO115" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="116" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A116" s="6" t="s">
         <v>485</v>
       </c>
@@ -22230,8 +22612,11 @@
         <f t="shared" si="19"/>
         <v>0.6706877524292354</v>
       </c>
+      <c r="AO116" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="117" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A117" s="6" t="s">
         <v>485</v>
       </c>
@@ -22351,8 +22736,11 @@
         <f t="shared" si="19"/>
         <v>0.64075267145675929</v>
       </c>
+      <c r="AO117" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="118" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A118" s="6" t="s">
         <v>485</v>
       </c>
@@ -22472,8 +22860,11 @@
         <f t="shared" si="19"/>
         <v>0.61151467271213211</v>
       </c>
+      <c r="AO118" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="119" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A119" s="6" t="s">
         <v>485</v>
       </c>
@@ -22593,8 +22984,11 @@
         <f t="shared" si="19"/>
         <v>1.9492775508164899</v>
       </c>
+      <c r="AO119" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="120" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A120" s="6" t="s">
         <v>486</v>
       </c>
@@ -22714,8 +23108,11 @@
         <f t="shared" si="19"/>
         <v>1.2292115404911319</v>
       </c>
+      <c r="AO120" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="121" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A121" s="6" t="s">
         <v>487</v>
       </c>
@@ -22835,8 +23232,11 @@
         <f t="shared" si="19"/>
         <v>1.2413630323963301</v>
       </c>
+      <c r="AO121" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="122" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A122" s="6" t="s">
         <v>488</v>
       </c>
@@ -22956,8 +23356,11 @@
         <f t="shared" si="19"/>
         <v>1.2561653093904881</v>
       </c>
+      <c r="AO122" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="123" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A123" s="6" t="s">
         <v>489</v>
       </c>
@@ -23077,8 +23480,11 @@
         <f t="shared" si="19"/>
         <v>1.2113560025023844</v>
       </c>
+      <c r="AO123" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="124" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A124" s="6" t="s">
         <v>490</v>
       </c>
@@ -23198,8 +23604,11 @@
         <f t="shared" si="19"/>
         <v>2.613496932515337</v>
       </c>
+      <c r="AO124" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="125" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A125" s="6" t="s">
         <v>490</v>
       </c>
@@ -23319,8 +23728,11 @@
         <f t="shared" si="19"/>
         <v>2.6134969325153379</v>
       </c>
+      <c r="AO125" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="126" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A126" s="6" t="s">
         <v>491</v>
       </c>
@@ -23440,8 +23852,11 @@
         <f t="shared" si="19"/>
         <v>1.3821716627734322</v>
       </c>
+      <c r="AO126" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="127" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A127" s="6" t="s">
         <v>492</v>
       </c>
@@ -23561,8 +23976,11 @@
         <f t="shared" si="19"/>
         <v>1.3508286832235206</v>
       </c>
+      <c r="AO127" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="128" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A128" s="6" t="s">
         <v>492</v>
       </c>
@@ -23682,8 +24100,11 @@
         <f t="shared" si="19"/>
         <v>1.3273996567144928</v>
       </c>
+      <c r="AO128" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="129" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A129" s="6" t="s">
         <v>520</v>
       </c>
@@ -23803,8 +24224,11 @@
         <f t="shared" si="19"/>
         <v>1.6857797571068185</v>
       </c>
+      <c r="AO129" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="130" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A130" s="6" t="s">
         <v>494</v>
       </c>
@@ -23924,8 +24348,11 @@
         <f t="shared" si="19"/>
         <v>1.1873209657838852</v>
       </c>
+      <c r="AO130" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="131" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A131" s="6" t="s">
         <v>494</v>
       </c>
@@ -24045,8 +24472,11 @@
         <f t="shared" ref="AN131:AN194" si="29">AI131*AM131/(AD131+AB131)</f>
         <v>1.1478379123898732</v>
       </c>
+      <c r="AO131" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="132" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A132" s="6" t="s">
         <v>495</v>
       </c>
@@ -24166,8 +24596,11 @@
         <f t="shared" si="29"/>
         <v>1.1697737528257561</v>
       </c>
+      <c r="AO132" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="133" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A133" s="6" t="s">
         <v>520</v>
       </c>
@@ -24287,8 +24720,11 @@
         <f t="shared" si="29"/>
         <v>1.6461735009491525</v>
       </c>
+      <c r="AO133" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="134" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A134" s="6" t="s">
         <v>497</v>
       </c>
@@ -24408,8 +24844,11 @@
         <f t="shared" si="29"/>
         <v>1.1917791466511929</v>
       </c>
+      <c r="AO134" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="135" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A135" s="6" t="s">
         <v>497</v>
       </c>
@@ -24529,8 +24968,11 @@
         <f t="shared" si="29"/>
         <v>1.1697737528257561</v>
       </c>
+      <c r="AO135" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="136" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A136" s="6" t="s">
         <v>497</v>
       </c>
@@ -24650,8 +25092,11 @@
         <f t="shared" si="29"/>
         <v>1.1478379123898732</v>
       </c>
+      <c r="AO136" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="137" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A137" s="6" t="s">
         <v>498</v>
       </c>
@@ -24770,8 +25215,11 @@
         <f t="shared" si="29"/>
         <v>1.100201380402013</v>
       </c>
+      <c r="AO137" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="138" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A138" s="6" t="s">
         <v>498</v>
       </c>
@@ -24885,8 +25333,11 @@
         <f t="shared" si="29"/>
         <v>3.4285714285714284</v>
       </c>
+      <c r="AO138" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="139" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A139" s="6" t="s">
         <v>498</v>
       </c>
@@ -25005,8 +25456,11 @@
         <f t="shared" si="29"/>
         <v>1.5534532233799874</v>
       </c>
+      <c r="AO139" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="140" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A140" s="6" t="s">
         <v>498</v>
       </c>
@@ -25120,8 +25574,11 @@
         <f t="shared" si="29"/>
         <v>3.4285714285714284</v>
       </c>
+      <c r="AO140" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="141" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A141" s="6" t="s">
         <v>499</v>
       </c>
@@ -25241,8 +25698,11 @@
         <f t="shared" si="29"/>
         <v>1.3402722285622568</v>
       </c>
+      <c r="AO141" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="142" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A142" s="6" t="s">
         <v>499</v>
       </c>
@@ -25362,8 +25822,11 @@
         <f t="shared" si="29"/>
         <v>1.1069472501692708</v>
       </c>
+      <c r="AO142" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="143" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A143" s="6" t="s">
         <v>499</v>
       </c>
@@ -25483,8 +25946,11 @@
         <f t="shared" si="29"/>
         <v>1.3096934841312509</v>
       </c>
+      <c r="AO143" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="144" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A144" s="6" t="s">
         <v>500</v>
       </c>
@@ -25604,8 +26070,11 @@
         <f t="shared" si="29"/>
         <v>1.2649802836537249</v>
       </c>
+      <c r="AO144" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="145" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A145" s="6" t="s">
         <v>501</v>
       </c>
@@ -25725,8 +26194,11 @@
         <f t="shared" si="29"/>
         <v>1.242648133063637</v>
       </c>
+      <c r="AO145" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="146" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A146" s="6" t="s">
         <v>502</v>
       </c>
@@ -25846,8 +26318,11 @@
         <f t="shared" si="29"/>
         <v>0.90074899958421728</v>
       </c>
+      <c r="AO146" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="147" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A147" s="6" t="s">
         <v>502</v>
       </c>
@@ -25967,8 +26442,11 @@
         <f t="shared" si="29"/>
         <v>0.86471997316517379</v>
       </c>
+      <c r="AO147" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="148" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A148" s="6" t="s">
         <v>502</v>
       </c>
@@ -26088,8 +26566,11 @@
         <f t="shared" si="29"/>
         <v>0.8291908931927453</v>
       </c>
+      <c r="AO148" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="149" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A149" s="6" t="s">
         <v>502</v>
       </c>
@@ -26209,8 +26690,11 @@
         <f t="shared" si="29"/>
         <v>0.82391222601076908</v>
       </c>
+      <c r="AO149" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="150" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A150" s="6" t="s">
         <v>502</v>
       </c>
@@ -26330,8 +26814,11 @@
         <f t="shared" si="29"/>
         <v>1.307592918802565</v>
       </c>
+      <c r="AO150" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="151" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A151" s="6" t="s">
         <v>502</v>
       </c>
@@ -26451,8 +26938,11 @@
         <f t="shared" si="29"/>
         <v>1.259710619839457</v>
       </c>
+      <c r="AO151" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="152" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A152" s="6" t="s">
         <v>502</v>
       </c>
@@ -26566,8 +27056,11 @@
         <f t="shared" si="29"/>
         <v>2</v>
       </c>
+      <c r="AO152" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="153" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A153" s="6" t="s">
         <v>502</v>
       </c>
@@ -26687,8 +27180,11 @@
         <f t="shared" si="29"/>
         <v>1.5199940748831153</v>
       </c>
+      <c r="AO153" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="154" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A154" s="6" t="s">
         <v>502</v>
       </c>
@@ -26808,8 +27304,11 @@
         <f t="shared" si="29"/>
         <v>0.94841385595929528</v>
       </c>
+      <c r="AO154" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="155" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A155" s="6" t="s">
         <v>503</v>
       </c>
@@ -26929,8 +27428,11 @@
         <f t="shared" si="29"/>
         <v>2.001711919813113</v>
       </c>
+      <c r="AO155" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="156" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A156" s="6" t="s">
         <v>503</v>
       </c>
@@ -27050,8 +27552,11 @@
         <f t="shared" si="29"/>
         <v>2.7873981870831179</v>
       </c>
+      <c r="AO156" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="157" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A157" s="6" t="s">
         <v>503</v>
       </c>
@@ -27171,8 +27676,11 @@
         <f t="shared" si="29"/>
         <v>1.8835744163813872</v>
       </c>
+      <c r="AO157" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="158" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A158" s="6" t="s">
         <v>548</v>
       </c>
@@ -27292,8 +27800,11 @@
         <f t="shared" si="29"/>
         <v>1.3178084967631456</v>
       </c>
+      <c r="AO158" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="159" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A159" s="6" t="s">
         <v>547</v>
       </c>
@@ -27413,8 +27924,11 @@
         <f t="shared" si="29"/>
         <v>1.3730404099510281</v>
       </c>
+      <c r="AO159" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="160" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A160" s="6" t="s">
         <v>504</v>
       </c>
@@ -27534,8 +28048,11 @@
         <f t="shared" si="29"/>
         <v>1.3848749369337743</v>
       </c>
+      <c r="AO160" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="161" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A161" s="6" t="s">
         <v>505</v>
       </c>
@@ -27655,8 +28172,11 @@
         <f t="shared" si="29"/>
         <v>1.3585676614027813</v>
       </c>
+      <c r="AO161" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="162" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A162" s="6" t="s">
         <v>506</v>
       </c>
@@ -27776,8 +28296,11 @@
         <f t="shared" si="29"/>
         <v>1.372740519264412</v>
       </c>
+      <c r="AO162" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="163" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A163" s="6" t="s">
         <v>507</v>
       </c>
@@ -27897,8 +28420,11 @@
         <f t="shared" si="29"/>
         <v>1.3209122633460484</v>
       </c>
+      <c r="AO163" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="164" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A164" s="6" t="s">
         <v>508</v>
       </c>
@@ -28018,8 +28544,11 @@
         <f t="shared" si="29"/>
         <v>4.2857142857142856</v>
       </c>
+      <c r="AO164" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="165" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A165" s="6" t="s">
         <v>509</v>
       </c>
@@ -28139,8 +28668,11 @@
         <f t="shared" si="29"/>
         <v>0.89768559755339483</v>
       </c>
+      <c r="AO165" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="166" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A166" s="6" t="s">
         <v>510</v>
       </c>
@@ -28260,8 +28792,11 @@
         <f t="shared" si="29"/>
         <v>0.84488056240319498</v>
       </c>
+      <c r="AO166" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="167" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A167" s="6" t="s">
         <v>511</v>
       </c>
@@ -28381,8 +28916,11 @@
         <f t="shared" si="29"/>
         <v>0.79115858344502654</v>
       </c>
+      <c r="AO167" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="168" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A168" s="6" t="s">
         <v>512</v>
       </c>
@@ -28502,8 +29040,11 @@
         <f t="shared" si="29"/>
         <v>0.77406888933587614</v>
       </c>
+      <c r="AO168" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="169" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A169" s="6" t="s">
         <v>513</v>
       </c>
@@ -28623,8 +29164,11 @@
         <f t="shared" si="29"/>
         <v>0.95007407159306967</v>
       </c>
+      <c r="AO169" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="170" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A170" s="6" t="s">
         <v>514</v>
       </c>
@@ -28744,8 +29288,11 @@
         <f t="shared" si="29"/>
         <v>1.6504684110205614</v>
       </c>
+      <c r="AO170" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="171" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A171" s="6" t="s">
         <v>514</v>
       </c>
@@ -28865,8 +29412,11 @@
         <f t="shared" si="29"/>
         <v>1.5959766651655141</v>
       </c>
+      <c r="AO171" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="172" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A172" s="6" t="s">
         <v>514</v>
       </c>
@@ -28986,8 +29536,11 @@
         <f t="shared" si="29"/>
         <v>1.541459129098488</v>
       </c>
+      <c r="AO172" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="173" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A173" s="6" t="s">
         <v>514</v>
       </c>
@@ -29107,8 +29660,11 @@
         <f t="shared" si="29"/>
         <v>1.4870446603133847</v>
       </c>
+      <c r="AO173" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="174" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A174" s="6" t="s">
         <v>515</v>
       </c>
@@ -29228,8 +29784,11 @@
         <f t="shared" si="29"/>
         <v>1.29803634535601</v>
       </c>
+      <c r="AO174" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="175" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A175" s="6" t="s">
         <v>516</v>
       </c>
@@ -29349,8 +29908,11 @@
         <f t="shared" si="29"/>
         <v>1.2979593269679877</v>
       </c>
+      <c r="AO175" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="176" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A176" s="6" t="s">
         <v>517</v>
       </c>
@@ -29470,8 +30032,11 @@
         <f t="shared" si="29"/>
         <v>1.6263477020219728</v>
       </c>
+      <c r="AO176" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="177" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A177" s="6" t="s">
         <v>518</v>
       </c>
@@ -29591,8 +30156,11 @@
         <f t="shared" si="29"/>
         <v>1.2592386722239013</v>
       </c>
+      <c r="AO177" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="178" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A178" s="6" t="s">
         <v>519</v>
       </c>
@@ -29712,8 +30280,11 @@
         <f t="shared" si="29"/>
         <v>1.4641218723147973</v>
       </c>
+      <c r="AO178" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="179" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A179" s="6" t="s">
         <v>521</v>
       </c>
@@ -29833,12 +30404,15 @@
         <f t="shared" si="29"/>
         <v>1.5931435361112869</v>
       </c>
+      <c r="AO179" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="180" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A180" s="6" t="s">
         <v>470</v>
       </c>
-      <c r="B180" s="53" t="s">
+      <c r="B180" s="6" t="s">
         <v>734</v>
       </c>
       <c r="C180" s="36" t="s">
@@ -29954,8 +30528,11 @@
         <f t="shared" si="29"/>
         <v>1.4269848890125221</v>
       </c>
+      <c r="AO180" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="181" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A181" s="6" t="s">
         <v>535</v>
       </c>
@@ -30075,8 +30652,11 @@
         <f t="shared" si="29"/>
         <v>1.3995973831143944</v>
       </c>
+      <c r="AO181" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="182" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A182" s="6" t="s">
         <v>522</v>
       </c>
@@ -30196,8 +30776,11 @@
         <f t="shared" si="29"/>
         <v>1.4757143571699876</v>
       </c>
+      <c r="AO182" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="183" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A183" s="6" t="s">
         <v>522</v>
       </c>
@@ -30317,8 +30900,11 @@
         <f t="shared" si="29"/>
         <v>1.4374300869105257</v>
       </c>
+      <c r="AO183" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="184" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A184" s="6" t="s">
         <v>522</v>
       </c>
@@ -30438,8 +31024,11 @@
         <f t="shared" si="29"/>
         <v>1.3985631033192503</v>
       </c>
+      <c r="AO184" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="185" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A185" s="6" t="s">
         <v>523</v>
       </c>
@@ -30559,8 +31148,11 @@
         <f t="shared" si="29"/>
         <v>1.3826456374022646</v>
       </c>
+      <c r="AO185" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="186" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A186" s="6" t="s">
         <v>524</v>
       </c>
@@ -30680,8 +31272,11 @@
         <f t="shared" si="29"/>
         <v>0.47357002940963111</v>
       </c>
+      <c r="AO186" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="187" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A187" s="6" t="s">
         <v>525</v>
       </c>
@@ -30801,8 +31396,11 @@
         <f t="shared" si="29"/>
         <v>1.2597354394053424</v>
       </c>
+      <c r="AO187" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="188" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A188" s="6" t="s">
         <v>526</v>
       </c>
@@ -30922,8 +31520,11 @@
         <f t="shared" si="29"/>
         <v>1.1675517449568096</v>
       </c>
+      <c r="AO188" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="189" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A189" s="6" t="s">
         <v>527</v>
       </c>
@@ -31043,8 +31644,11 @@
         <f t="shared" si="29"/>
         <v>1.3696411756979359</v>
       </c>
+      <c r="AO189" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="190" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A190" s="6" t="s">
         <v>527</v>
       </c>
@@ -31164,8 +31768,11 @@
         <f t="shared" si="29"/>
         <v>1.350214188462304</v>
       </c>
+      <c r="AO190" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="191" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A191" s="6" t="s">
         <v>528</v>
       </c>
@@ -31285,8 +31892,11 @@
         <f t="shared" si="29"/>
         <v>1.2329454023052526</v>
       </c>
+      <c r="AO191" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="192" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A192" s="6" t="s">
         <v>528</v>
       </c>
@@ -31406,8 +32016,11 @@
         <f t="shared" si="29"/>
         <v>1.1957801977735603</v>
       </c>
+      <c r="AO192" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="193" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A193" s="6" t="s">
         <v>529</v>
       </c>
@@ -31527,8 +32140,11 @@
         <f t="shared" si="29"/>
         <v>1.1035853568830785</v>
       </c>
+      <c r="AO193" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="194" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A194" s="6" t="s">
         <v>529</v>
       </c>
@@ -31606,7 +32222,7 @@
         <v>39.066288080668613</v>
       </c>
       <c r="AC194" s="20">
-        <f t="shared" ref="AC194:AC237" si="33">IF(AI194=0,0,AB194/AI194)</f>
+        <f t="shared" ref="AC194:AC236" si="33">IF(AI194=0,0,AB194/AI194)</f>
         <v>0.33668194854700417</v>
       </c>
       <c r="AD194" s="21">
@@ -31641,15 +32257,18 @@
         <v>43225.410942956936</v>
       </c>
       <c r="AM194" s="2">
-        <f t="shared" ref="AM194:AM242" si="38">Q194+X194</f>
+        <f t="shared" ref="AM194:AM241" si="38">Q194+X194</f>
         <v>0.7</v>
       </c>
       <c r="AN194" s="51">
         <f t="shared" si="29"/>
         <v>1.0659650406849812</v>
       </c>
+      <c r="AO194" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="195" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A195" s="6" t="s">
         <v>529</v>
       </c>
@@ -31769,8 +32388,11 @@
         <f t="shared" ref="AN195:AN239" si="39">AI195*AM195/(AD195+AB195)</f>
         <v>2.1875</v>
       </c>
+      <c r="AO195" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="196" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A196" s="6" t="s">
         <v>529</v>
       </c>
@@ -31890,8 +32512,11 @@
         <f t="shared" si="39"/>
         <v>2.1875</v>
       </c>
+      <c r="AO196" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="197" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A197" s="6" t="s">
         <v>529</v>
       </c>
@@ -32011,8 +32636,11 @@
         <f t="shared" si="39"/>
         <v>2.1875</v>
       </c>
+      <c r="AO197" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="198" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A198" s="6" t="s">
         <v>529</v>
       </c>
@@ -32132,8 +32760,11 @@
         <f t="shared" si="39"/>
         <v>2.1875</v>
       </c>
+      <c r="AO198" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="199" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A199" s="6" t="s">
         <v>529</v>
       </c>
@@ -32253,8 +32884,11 @@
         <f t="shared" si="39"/>
         <v>2.1875</v>
       </c>
+      <c r="AO199" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="200" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A200" s="6" t="s">
         <v>529</v>
       </c>
@@ -32374,8 +33008,11 @@
         <f t="shared" si="39"/>
         <v>2.1875</v>
       </c>
+      <c r="AO200" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="201" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A201" s="6" t="s">
         <v>530</v>
       </c>
@@ -32494,8 +33131,11 @@
         <f t="shared" si="39"/>
         <v>1.6566885721095854</v>
       </c>
+      <c r="AO201" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="202" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A202" s="6" t="s">
         <v>530</v>
       </c>
@@ -32614,8 +33254,11 @@
         <f t="shared" si="39"/>
         <v>1.6346161037144891</v>
       </c>
+      <c r="AO202" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="203" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A203" s="6" t="s">
         <v>531</v>
       </c>
@@ -32734,8 +33377,11 @@
         <f t="shared" si="39"/>
         <v>1.5890770411330262</v>
       </c>
+      <c r="AO203" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="204" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A204" s="6" t="s">
         <v>532</v>
       </c>
@@ -32855,8 +33501,11 @@
         <f t="shared" si="39"/>
         <v>1.6348488056211639</v>
       </c>
+      <c r="AO204" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="205" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A205" s="6" t="s">
         <v>533</v>
       </c>
@@ -32976,8 +33625,11 @@
         <f t="shared" si="39"/>
         <v>1.3994784856987472</v>
       </c>
+      <c r="AO205" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="206" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A206" s="6" t="s">
         <v>533</v>
       </c>
@@ -33097,8 +33749,11 @@
         <f t="shared" si="39"/>
         <v>1.3761547970799959</v>
       </c>
+      <c r="AO206" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="207" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A207" s="6" t="s">
         <v>534</v>
       </c>
@@ -33218,8 +33873,11 @@
         <f t="shared" si="39"/>
         <v>1.2739382867033264</v>
       </c>
+      <c r="AO207" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="208" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A208" s="6" t="s">
         <v>534</v>
       </c>
@@ -33339,8 +33997,11 @@
         <f t="shared" si="39"/>
         <v>1.2513432560545719</v>
       </c>
+      <c r="AO208" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="209" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A209" s="6" t="s">
         <v>534</v>
       </c>
@@ -33460,8 +34121,11 @@
         <f t="shared" si="39"/>
         <v>1.2287862611479596</v>
       </c>
+      <c r="AO209" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="210" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A210" s="6" t="s">
         <v>534</v>
       </c>
@@ -33581,8 +34245,11 @@
         <f t="shared" si="39"/>
         <v>1.1838391039622553</v>
       </c>
+      <c r="AO210" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="211" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A211" s="6" t="s">
         <v>535</v>
       </c>
@@ -33702,8 +34369,11 @@
         <f t="shared" si="39"/>
         <v>1.4269474786562346</v>
       </c>
+      <c r="AO211" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="212" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A212" s="6" t="s">
         <v>536</v>
       </c>
@@ -33823,8 +34493,11 @@
         <f t="shared" si="39"/>
         <v>1.4544075393871425</v>
       </c>
+      <c r="AO212" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="213" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A213" s="28" t="s">
         <v>579</v>
       </c>
@@ -33858,7 +34531,7 @@
       <c r="O213" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="P213" s="37"/>
+      <c r="P213" s="45"/>
       <c r="Q213" s="29">
         <v>0.7</v>
       </c>
@@ -33924,8 +34597,11 @@
         <f t="shared" si="39"/>
         <v>#DIV/0!</v>
       </c>
+      <c r="AO213" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="214" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A214" s="6" t="s">
         <v>537</v>
       </c>
@@ -34045,8 +34721,11 @@
         <f t="shared" si="39"/>
         <v>1.1915152802141717</v>
       </c>
+      <c r="AO214" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="215" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A215" s="6" t="s">
         <v>538</v>
       </c>
@@ -34165,8 +34844,11 @@
         <f t="shared" si="39"/>
         <v>1.3027775635825822</v>
       </c>
+      <c r="AO215" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="216" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A216" s="6" t="s">
         <v>539</v>
       </c>
@@ -34285,8 +34967,11 @@
         <f t="shared" si="39"/>
         <v>0.81407876134588997</v>
       </c>
+      <c r="AO216" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="217" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A217" s="6" t="s">
         <v>540</v>
       </c>
@@ -34405,8 +35090,11 @@
         <f t="shared" si="39"/>
         <v>1.1216996276148128</v>
       </c>
+      <c r="AO217" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="218" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A218" s="6" t="s">
         <v>541</v>
       </c>
@@ -34526,8 +35214,11 @@
         <f t="shared" si="39"/>
         <v>1.1919024331549293</v>
       </c>
+      <c r="AO218" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="219" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A219" s="6" t="s">
         <v>542</v>
       </c>
@@ -34647,8 +35338,11 @@
         <f t="shared" si="39"/>
         <v>0</v>
       </c>
+      <c r="AO219" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="220" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A220" s="6" t="s">
         <v>433</v>
       </c>
@@ -34768,8 +35462,11 @@
         <f t="shared" si="39"/>
         <v>1.4778743985473446</v>
       </c>
+      <c r="AO220" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="221" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A221" s="6" t="s">
         <v>433</v>
       </c>
@@ -34889,8 +35586,11 @@
         <f t="shared" si="39"/>
         <v>1.4352282729652679</v>
       </c>
+      <c r="AO221" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="222" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A222" s="6" t="s">
         <v>543</v>
       </c>
@@ -35004,8 +35704,11 @@
         <f t="shared" si="39"/>
         <v>2.6923076923076925</v>
       </c>
+      <c r="AO222" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="223" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A223" s="6" t="s">
         <v>544</v>
       </c>
@@ -35119,8 +35822,11 @@
         <f t="shared" si="39"/>
         <v>3.378378378378379</v>
       </c>
+      <c r="AO223" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="224" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A224" s="6" t="s">
         <v>544</v>
       </c>
@@ -35234,8 +35940,11 @@
         <f t="shared" si="39"/>
         <v>3.378378378378379</v>
       </c>
+      <c r="AO224" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="225" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A225" s="6" t="s">
         <v>544</v>
       </c>
@@ -35349,8 +36058,11 @@
         <f t="shared" si="39"/>
         <v>3.3783783783783781</v>
       </c>
+      <c r="AO225" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="226" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A226" s="6" t="s">
         <v>544</v>
       </c>
@@ -35464,8 +36176,11 @@
         <f t="shared" si="39"/>
         <v>3.3783783783783781</v>
       </c>
+      <c r="AO226" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="227" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A227" s="6" t="s">
         <v>544</v>
       </c>
@@ -35579,8 +36294,11 @@
         <f t="shared" si="39"/>
         <v>3.3783783783783781</v>
       </c>
+      <c r="AO227" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="228" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A228" s="6" t="s">
         <v>544</v>
       </c>
@@ -35694,8 +36412,11 @@
         <f t="shared" si="39"/>
         <v>3.3783783783783785</v>
       </c>
+      <c r="AO228" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="229" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A229" s="6" t="s">
         <v>544</v>
       </c>
@@ -35809,8 +36530,11 @@
         <f t="shared" si="39"/>
         <v>3.3783783783783781</v>
       </c>
+      <c r="AO229" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="230" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A230" s="6" t="s">
         <v>544</v>
       </c>
@@ -35924,8 +36648,11 @@
         <f t="shared" si="39"/>
         <v>3.3783783783783785</v>
       </c>
+      <c r="AO230" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="231" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A231" s="28" t="s">
         <v>575</v>
       </c>
@@ -36020,7 +36747,7 @@
         <v>723899.17</v>
       </c>
       <c r="AL231" s="22">
-        <f t="shared" ref="AL231:AL242" si="42">AE231*AF231</f>
+        <f t="shared" ref="AL231:AL241" si="42">AE231*AF231</f>
         <v>0</v>
       </c>
       <c r="AM231" s="2">
@@ -36031,8 +36758,11 @@
         <f t="shared" si="39"/>
         <v>#DIV/0!</v>
       </c>
+      <c r="AO231" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="232" spans="1:40" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:41" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A232" s="31" t="s">
         <v>576</v>
       </c>
@@ -36134,8 +36864,11 @@
         <f t="shared" si="39"/>
         <v>#DIV/0!</v>
       </c>
+      <c r="AO232" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="233" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A233" s="6" t="s">
         <v>584</v>
       </c>
@@ -36169,7 +36902,7 @@
       <c r="O233" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="P233" s="37">
+      <c r="P233" s="45">
         <v>2029</v>
       </c>
       <c r="Q233" s="29">
@@ -36237,8 +36970,11 @@
         <f t="shared" si="39"/>
         <v>#DIV/0!</v>
       </c>
+      <c r="AO233" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="234" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A234" s="28" t="s">
         <v>577</v>
       </c>
@@ -36272,7 +37008,7 @@
       <c r="O234" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="P234" s="37"/>
+      <c r="P234" s="45"/>
       <c r="Q234" s="29">
         <v>0.8</v>
       </c>
@@ -36340,8 +37076,11 @@
         <f t="shared" si="39"/>
         <v>2.2839969947407965</v>
       </c>
+      <c r="AO234" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="235" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A235" s="28" t="s">
         <v>578</v>
       </c>
@@ -36375,7 +37114,7 @@
       <c r="O235" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="P235" s="37"/>
+      <c r="P235" s="45"/>
       <c r="Q235" s="29">
         <v>0.7</v>
       </c>
@@ -36441,8 +37180,11 @@
         <f t="shared" si="39"/>
         <v>#DIV/0!</v>
       </c>
+      <c r="AO235" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="236" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A236" s="28" t="s">
         <v>580</v>
       </c>
@@ -36476,7 +37218,7 @@
       <c r="O236" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="P236" s="37"/>
+      <c r="P236" s="45"/>
       <c r="Q236" s="29">
         <v>0.7</v>
       </c>
@@ -36542,8 +37284,11 @@
         <f t="shared" si="39"/>
         <v>#DIV/0!</v>
       </c>
+      <c r="AO236" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="237" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A237" s="6" t="s">
         <v>496</v>
       </c>
@@ -36663,8 +37408,11 @@
         <f t="shared" si="39"/>
         <v>1.1478379123898734</v>
       </c>
+      <c r="AO237" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="238" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A238" s="28" t="s">
         <v>581</v>
       </c>
@@ -36696,7 +37444,7 @@
         <v>613</v>
       </c>
       <c r="O238" s="6"/>
-      <c r="P238" s="37">
+      <c r="P238" s="45">
         <v>2026</v>
       </c>
       <c r="Q238" s="29">
@@ -36706,7 +37454,7 @@
         <v>0.2</v>
       </c>
       <c r="S238" s="40">
-        <f t="shared" ref="S238:S242" si="43">SUM(Q238:R238)</f>
+        <f t="shared" ref="S238:S244" si="43">SUM(Q238:R238)</f>
         <v>1</v>
       </c>
       <c r="T238" s="37"/>
@@ -36724,11 +37472,11 @@
         <v>0</v>
       </c>
       <c r="AC238" s="20">
-        <f t="shared" ref="AC238:AC240" si="45">IF(AI238=0,0,AB238/AI238)</f>
+        <f t="shared" ref="AC238:AC244" si="45">IF(AI238=0,0,AB238/AI238)</f>
         <v>0</v>
       </c>
       <c r="AD238" s="21">
-        <f t="shared" ref="AD238:AD240" si="46">(AE238*AF238*AG238)/10^6</f>
+        <f t="shared" ref="AD238:AD244" si="46">(AE238*AF238*AG238)/10^6</f>
         <v>53.243993000000003</v>
       </c>
       <c r="AE238" s="13">
@@ -36744,11 +37492,11 @@
         <v>540</v>
       </c>
       <c r="AI238" s="21">
-        <f t="shared" ref="AI238:AI242" si="47">(AH238*AG238*AF238)/10^6</f>
+        <f t="shared" ref="AI238:AI241" si="47">(AH238*AG238*AF238)/10^6</f>
         <v>216.0162</v>
       </c>
       <c r="AJ238" s="21">
-        <f t="shared" ref="AJ238:AJ242" si="48">AI238*Q238</f>
+        <f t="shared" ref="AJ238:AJ241" si="48">AI238*Q238</f>
         <v>172.81296</v>
       </c>
       <c r="AK238" s="30">
@@ -36766,8 +37514,11 @@
         <f t="shared" si="39"/>
         <v>3.2456799398948157</v>
       </c>
+      <c r="AO238" s="75" t="s">
+        <v>789</v>
+      </c>
     </row>
-    <row r="239" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A239" s="28" t="s">
         <v>582</v>
       </c>
@@ -36801,7 +37552,7 @@
       <c r="O239" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="P239" s="37"/>
+      <c r="P239" s="45"/>
       <c r="Q239" s="47">
         <v>0.8</v>
       </c>
@@ -36867,8 +37618,11 @@
         <f t="shared" si="39"/>
         <v>#DIV/0!</v>
       </c>
+      <c r="AO239" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="240" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A240" s="28" t="s">
         <v>583</v>
       </c>
@@ -36902,7 +37656,7 @@
       <c r="O240" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="P240" s="6"/>
+      <c r="P240" s="77"/>
       <c r="Q240" s="47">
         <v>0.72</v>
       </c>
@@ -36968,8 +37722,11 @@
         <f>AI240*AM240/(AD240+AB240)</f>
         <v>#DIV/0!</v>
       </c>
+      <c r="AO240" s="75" t="s">
+        <v>788</v>
+      </c>
     </row>
-    <row r="241" spans="1:40" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:41" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A241" s="6" t="s">
         <v>587</v>
       </c>
@@ -37001,7 +37758,7 @@
       <c r="O241" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="P241" s="37"/>
+      <c r="P241" s="45"/>
       <c r="Q241" s="47">
         <v>0.72499999999999998</v>
       </c>
@@ -37022,9 +37779,17 @@
       <c r="AA241" s="19">
         <v>1669.242</v>
       </c>
-      <c r="AB241" s="37"/>
-      <c r="AC241" s="37"/>
-      <c r="AD241" s="37"/>
+      <c r="AB241" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC241" s="20">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="AD241" s="21">
+        <f>(AE241*AF241*AG241)/10^6</f>
+        <v>196.54908</v>
+      </c>
       <c r="AE241" s="13">
         <v>240</v>
       </c>
@@ -37056,23 +37821,28 @@
         <f t="shared" si="38"/>
         <v>0.72499999999999998</v>
       </c>
-      <c r="AN241" s="51" t="e">
+      <c r="AN241" s="51">
         <f>AI241*AM241/(AD241+AB241)</f>
-        <v>#DIV/0!</v>
+        <v>1.5708333333333331</v>
+      </c>
+      <c r="AO241" s="75" t="s">
+        <v>789</v>
       </c>
     </row>
-    <row r="242" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A242" s="6" t="s">
         <v>785</v>
       </c>
       <c r="B242" s="6" t="s">
         <v>782</v>
       </c>
-      <c r="D242" s="12"/>
-      <c r="E242" s="74"/>
-      <c r="F242" s="74"/>
-      <c r="G242" s="74"/>
-      <c r="H242" s="74"/>
+      <c r="D242" s="12">
+        <v>1</v>
+      </c>
+      <c r="E242" s="73"/>
+      <c r="F242" s="73"/>
+      <c r="G242" s="73"/>
+      <c r="H242" s="73"/>
       <c r="I242" s="37"/>
       <c r="J242" s="34" t="s">
         <v>598</v>
@@ -37092,7 +37862,7 @@
       <c r="O242" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="P242" s="37" t="s">
+      <c r="P242" s="45" t="s">
         <v>28</v>
       </c>
       <c r="Q242" s="47">
@@ -37105,19 +37875,27 @@
         <f t="shared" si="43"/>
         <v>1</v>
       </c>
-      <c r="T242" s="73"/>
-      <c r="U242" s="73"/>
-      <c r="V242" s="73"/>
-      <c r="W242" s="73"/>
-      <c r="X242" s="73"/>
-      <c r="Y242" s="73"/>
-      <c r="Z242" s="73"/>
+      <c r="T242" s="72"/>
+      <c r="U242" s="72"/>
+      <c r="V242" s="72"/>
+      <c r="W242" s="72"/>
+      <c r="X242" s="72"/>
+      <c r="Y242" s="72"/>
+      <c r="Z242" s="72"/>
       <c r="AA242" s="19">
         <v>184681</v>
       </c>
-      <c r="AB242" s="73"/>
-      <c r="AC242" s="20"/>
-      <c r="AD242" s="21"/>
+      <c r="AB242" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC242" s="20">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="AD242" s="21">
+        <f>(AE242*AF242*AG242)/10^6</f>
+        <v>72.25</v>
+      </c>
       <c r="AE242" s="13">
         <v>500</v>
       </c>
@@ -37149,13 +37927,224 @@
         <f>Q242+X242</f>
         <v>0.56999999999999995</v>
       </c>
-      <c r="AN242" s="51" t="e">
+      <c r="AN242" s="51">
         <f>AI242*AM242/(AD242+AB242)</f>
+        <v>3.9899999999999998</v>
+      </c>
+      <c r="AO242" s="75" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="243" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="A243" s="6" t="s">
+        <v>793</v>
+      </c>
+      <c r="B243" s="6" t="s">
+        <v>786</v>
+      </c>
+      <c r="D243" s="12">
+        <v>1</v>
+      </c>
+      <c r="E243" s="73"/>
+      <c r="F243" s="73"/>
+      <c r="G243" s="73"/>
+      <c r="H243" s="73"/>
+      <c r="I243" s="72"/>
+      <c r="J243" s="34" t="s">
+        <v>603</v>
+      </c>
+      <c r="K243" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="L243" s="6" t="s">
+        <v>790</v>
+      </c>
+      <c r="M243" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="N243" s="11" t="s">
+        <v>613</v>
+      </c>
+      <c r="O243" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P243" s="77" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q243" s="47">
+        <v>0.75</v>
+      </c>
+      <c r="R243" s="47">
+        <v>0.25</v>
+      </c>
+      <c r="S243" s="40">
+        <f t="shared" si="43"/>
+        <v>1</v>
+      </c>
+      <c r="T243" s="72"/>
+      <c r="U243" s="72"/>
+      <c r="V243" s="72"/>
+      <c r="W243" s="72"/>
+      <c r="X243" s="72"/>
+      <c r="Y243" s="72"/>
+      <c r="Z243" s="72"/>
+      <c r="AA243" s="79">
+        <v>780000</v>
+      </c>
+      <c r="AB243" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC243" s="20">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="AD243" s="21">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="AE243" s="72"/>
+      <c r="AF243" s="48">
+        <v>200</v>
+      </c>
+      <c r="AG243" s="48">
+        <v>2145</v>
+      </c>
+      <c r="AH243" s="48">
+        <v>550</v>
+      </c>
+      <c r="AI243" s="49">
+        <f t="shared" ref="AI243:AI244" si="49">(AH243*AG243*AF243)/10^6</f>
+        <v>235.95</v>
+      </c>
+      <c r="AJ243" s="21">
+        <f t="shared" ref="AJ243:AJ244" si="50">AI243*Q243</f>
+        <v>176.96249999999998</v>
+      </c>
+      <c r="AK243" s="30">
+        <v>110000</v>
+      </c>
+      <c r="AL243" s="22">
+        <f t="shared" ref="AL243:AL244" si="51">AE243*AF243</f>
+        <v>0</v>
+      </c>
+      <c r="AM243" s="2">
+        <f t="shared" ref="AM243:AM244" si="52">Q243+X243</f>
+        <v>0.75</v>
+      </c>
+      <c r="AN243" s="51" t="e">
+        <f>AI243*AM243/(AD243+AB243)</f>
         <v>#DIV/0!</v>
+      </c>
+      <c r="AO243" s="76" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="244" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="A244" s="6" t="s">
+        <v>794</v>
+      </c>
+      <c r="B244" s="6" t="s">
+        <v>791</v>
+      </c>
+      <c r="D244" s="12">
+        <v>1</v>
+      </c>
+      <c r="E244" s="73"/>
+      <c r="F244" s="73"/>
+      <c r="G244" s="73"/>
+      <c r="H244" s="73"/>
+      <c r="I244" s="72"/>
+      <c r="J244" s="34" t="s">
+        <v>599</v>
+      </c>
+      <c r="K244" s="6" t="s">
+        <v>792</v>
+      </c>
+      <c r="L244" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="M244" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="N244" s="11" t="s">
+        <v>613</v>
+      </c>
+      <c r="O244" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P244" s="78" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q244" s="47">
+        <v>0.67</v>
+      </c>
+      <c r="R244" s="47">
+        <v>0.33</v>
+      </c>
+      <c r="S244" s="40">
+        <f t="shared" si="43"/>
+        <v>1</v>
+      </c>
+      <c r="T244" s="72"/>
+      <c r="U244" s="72"/>
+      <c r="V244" s="72"/>
+      <c r="W244" s="72"/>
+      <c r="X244" s="72"/>
+      <c r="Y244" s="72"/>
+      <c r="Z244" s="72"/>
+      <c r="AA244" s="79">
+        <v>444727</v>
+      </c>
+      <c r="AB244" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC244" s="20">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="AD244" s="21">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="AE244" s="72"/>
+      <c r="AF244" s="48">
+        <v>250</v>
+      </c>
+      <c r="AG244" s="48">
+        <v>720</v>
+      </c>
+      <c r="AH244" s="48">
+        <v>700</v>
+      </c>
+      <c r="AI244" s="49">
+        <f>(AH244*AG244*AF244)/10^6</f>
+        <v>126</v>
+      </c>
+      <c r="AJ244" s="21">
+        <f>AI244*Q244</f>
+        <v>84.42</v>
+      </c>
+      <c r="AK244" s="30">
+        <v>175000</v>
+      </c>
+      <c r="AL244" s="22">
+        <f t="shared" si="51"/>
+        <v>0</v>
+      </c>
+      <c r="AM244" s="2">
+        <f t="shared" si="52"/>
+        <v>0.67</v>
+      </c>
+      <c r="AN244" s="51" t="e">
+        <f t="shared" ref="AN243:AN244" si="53">AI244*AM244/(AD244+AB244)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AO244" s="76" t="s">
+        <v>788</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK242" xr:uid="{9BB1E7F9-B7E0-4EE5-A96E-08F27078CA81}"/>
+  <autoFilter ref="A1:AK244" xr:uid="{9BB1E7F9-B7E0-4EE5-A96E-08F27078CA81}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C13" r:id="rId1" xr:uid="{20D620E2-00D1-4632-9A20-0409C8AFCC74}"/>
@@ -37224,17 +38213,17 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:26" x14ac:dyDescent="0.35">
-      <c r="C3" s="58" t="s">
+      <c r="C3" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="68" t="s">
+      <c r="D3" s="67" t="s">
         <v>745</v>
       </c>
-      <c r="O3" s="66"/>
-      <c r="P3" s="67" t="s">
+      <c r="O3" s="65"/>
+      <c r="P3" s="66" t="s">
         <v>753</v>
       </c>
-      <c r="Q3" s="67" t="s">
+      <c r="Q3" s="66" t="s">
         <v>754</v>
       </c>
     </row>
@@ -37247,39 +38236,39 @@
         <f t="array" ref="D4:D21">_xlfn.UNIQUE(AREAS!J2:J241)</f>
         <v>PA</v>
       </c>
-      <c r="F4" s="56" t="s">
+      <c r="F4" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="56">
+      <c r="G4" s="55">
         <f>COUNTA(_xlfn.ANCHORARRAY(C4))</f>
         <v>74</v>
       </c>
-      <c r="I4" s="56" t="s">
+      <c r="I4" s="55" t="s">
         <v>747</v>
       </c>
-      <c r="J4" s="57">
+      <c r="J4" s="56">
         <f>SUM(AREAS!AG2:AG1048576)</f>
-        <v>205570.0182683983</v>
-      </c>
-      <c r="L4" s="62" t="s">
+        <v>208435.0182683983</v>
+      </c>
+      <c r="L4" s="61" t="s">
         <v>748</v>
       </c>
-      <c r="M4" s="63">
+      <c r="M4" s="62">
         <f>M5/10000</f>
-        <v>5149.951158333477</v>
-      </c>
-      <c r="O4" s="56" t="s">
+        <v>5272.4238583334763</v>
+      </c>
+      <c r="O4" s="55" t="s">
         <v>751</v>
       </c>
-      <c r="P4" s="61">
+      <c r="P4" s="60">
         <f>SUM(AREAS!AI3:AI1048576)</f>
-        <v>33052.463694610124</v>
-      </c>
-      <c r="Q4" s="61">
+        <v>33414.413694610121</v>
+      </c>
+      <c r="Q4" s="60">
         <f>SUBTOTAL(9,AREAS!AI:AI)</f>
-        <v>33089.423694610115</v>
-      </c>
-      <c r="R4" s="55"/>
+        <v>33451.373694610113</v>
+      </c>
+      <c r="R4" s="54"/>
       <c r="T4" s="3">
         <f>COUNTA(T6:T77)</f>
         <v>72</v>
@@ -37292,49 +38281,49 @@
       <c r="D5" t="str">
         <v>SP</v>
       </c>
-      <c r="F5" s="56" t="s">
+      <c r="F5" s="55" t="s">
         <v>745</v>
       </c>
-      <c r="G5" s="56">
+      <c r="G5" s="55">
         <f>COUNTA(_xlfn.ANCHORARRAY(D4))</f>
         <v>18</v>
       </c>
-      <c r="L5" s="64" t="s">
+      <c r="L5" s="63" t="s">
         <v>749</v>
       </c>
-      <c r="M5" s="65">
+      <c r="M5" s="64">
         <f>SUM(AREAS!AA2:AA1048576)</f>
-        <v>51499511.583334766</v>
-      </c>
-      <c r="O5" s="56" t="s">
+        <v>52724238.583334766</v>
+      </c>
+      <c r="O5" s="55" t="s">
         <v>752</v>
       </c>
-      <c r="P5" s="61">
+      <c r="P5" s="60">
         <f>SUM(AREAS!AJ3:AJ1048576)</f>
-        <v>20751.134361209992</v>
-      </c>
-      <c r="Q5" s="61">
+        <v>21012.516861209991</v>
+      </c>
+      <c r="Q5" s="60">
         <f>SUBTOTAL(9,AREAS!AJ:AJ)</f>
-        <v>20788.094361209991</v>
-      </c>
-      <c r="R5" s="55"/>
-      <c r="T5" s="71" t="s">
+        <v>21049.476861209991</v>
+      </c>
+      <c r="R5" s="54"/>
+      <c r="T5" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="U5" s="71" t="s">
+      <c r="U5" s="70" t="s">
         <v>756</v>
       </c>
-      <c r="V5" s="71" t="s">
+      <c r="V5" s="70" t="s">
         <v>746</v>
       </c>
-      <c r="X5" s="69" t="s">
+      <c r="X5" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="Y5" s="70">
+      <c r="Y5" s="69">
         <f>COUNTIF(AREAS!L:L,Planilha2!X5)</f>
         <v>1</v>
       </c>
-      <c r="Z5" s="70">
+      <c r="Z5" s="69">
         <f>_xlfn.XLOOKUP(X5,AREAS!L:L,AREAS!D:D,"não")</f>
         <v>0</v>
       </c>
@@ -37346,7 +38335,7 @@
       <c r="D6" t="str">
         <v>TO</v>
       </c>
-      <c r="S6" s="72" t="s">
+      <c r="S6" s="71" t="s">
         <v>175</v>
       </c>
       <c r="T6" t="s">
@@ -37360,13 +38349,13 @@
         <f>_xlfn.XLOOKUP(T6,AREAS!L:L,AREAS!D:D,"não")</f>
         <v>1</v>
       </c>
-      <c r="X6" s="69" t="s">
+      <c r="X6" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="Y6" s="70">
+      <c r="Y6" s="69">
         <v>5</v>
       </c>
-      <c r="Z6" s="70">
+      <c r="Z6" s="69">
         <v>0</v>
       </c>
     </row>
@@ -37377,17 +38366,17 @@
       <c r="D7" t="str">
         <v>BA</v>
       </c>
-      <c r="E7" s="59" t="s">
+      <c r="E7" s="58" t="s">
         <v>588</v>
       </c>
-      <c r="F7" s="59">
+      <c r="F7" s="58">
         <v>0</v>
       </c>
       <c r="G7">
         <f>COUNTIF(AREAS!D:D,Planilha2!F7)</f>
         <v>8</v>
       </c>
-      <c r="S7" s="72" t="s">
+      <c r="S7" s="71" t="s">
         <v>95</v>
       </c>
       <c r="T7" t="s">
@@ -37401,14 +38390,14 @@
         <f>_xlfn.XLOOKUP(T7,AREAS!L:L,AREAS!D:D,"não")</f>
         <v>1</v>
       </c>
-      <c r="X7" s="69" t="s">
+      <c r="X7" s="68" t="s">
         <v>153</v>
       </c>
-      <c r="Y7" s="70">
+      <c r="Y7" s="69">
         <f>COUNTIF(AREAS!L:L,Planilha2!X7)</f>
         <v>2</v>
       </c>
-      <c r="Z7" s="70">
+      <c r="Z7" s="69">
         <f>_xlfn.XLOOKUP(X7,AREAS!L:L,AREAS!D:D,"não")</f>
         <v>0</v>
       </c>
@@ -37420,20 +38409,20 @@
       <c r="D8" t="str">
         <v>GO</v>
       </c>
-      <c r="E8" s="60" t="s">
+      <c r="E8" s="59" t="s">
         <v>746</v>
       </c>
-      <c r="F8" s="60">
+      <c r="F8" s="59">
         <v>1</v>
       </c>
       <c r="G8">
         <f>COUNTIF(AREAS!D:D,Planilha2!F8)</f>
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H8">
         <v>240</v>
       </c>
-      <c r="S8" s="72" t="s">
+      <c r="S8" s="71" t="s">
         <v>98</v>
       </c>
       <c r="T8" t="s">
@@ -37455,15 +38444,15 @@
       <c r="D9" t="str">
         <v>AL</v>
       </c>
-      <c r="F9" s="58" t="s">
+      <c r="F9" s="57" t="s">
         <v>750</v>
       </c>
-      <c r="G9" s="54">
+      <c r="G9" s="53">
         <f>SUM(G7:G8)</f>
-        <v>240</v>
-      </c>
-      <c r="P9" s="55"/>
-      <c r="S9" s="72" t="s">
+        <v>243</v>
+      </c>
+      <c r="P9" s="54"/>
+      <c r="S9" s="71" t="s">
         <v>103</v>
       </c>
       <c r="T9" t="s">
@@ -37485,8 +38474,8 @@
       <c r="D10" t="str">
         <v>PB</v>
       </c>
-      <c r="P10" s="55"/>
-      <c r="S10" s="72" t="s">
+      <c r="P10" s="54"/>
+      <c r="S10" s="71" t="s">
         <v>100</v>
       </c>
       <c r="T10" t="s">
@@ -37513,9 +38502,9 @@
       </c>
       <c r="G11">
         <f>G9</f>
-        <v>240</v>
-      </c>
-      <c r="S11" s="72" t="s">
+        <v>243</v>
+      </c>
+      <c r="S11" s="71" t="s">
         <v>757</v>
       </c>
       <c r="T11" t="s">
@@ -37537,7 +38526,7 @@
       <c r="D12" t="str">
         <v>CE</v>
       </c>
-      <c r="S12" s="72" t="s">
+      <c r="S12" s="71" t="s">
         <v>758</v>
       </c>
       <c r="T12" t="s">
@@ -37559,7 +38548,7 @@
       <c r="D13" t="str">
         <v>MA</v>
       </c>
-      <c r="S13" s="72" t="s">
+      <c r="S13" s="71" t="s">
         <v>90</v>
       </c>
       <c r="T13" t="s">
@@ -37581,7 +38570,7 @@
       <c r="D14" t="str">
         <v>MG</v>
       </c>
-      <c r="S14" s="72" t="s">
+      <c r="S14" s="71" t="s">
         <v>109</v>
       </c>
       <c r="T14" t="s">
@@ -37603,7 +38592,7 @@
       <c r="D15" t="str">
         <v>RJ</v>
       </c>
-      <c r="S15" s="72" t="s">
+      <c r="S15" s="71" t="s">
         <v>111</v>
       </c>
       <c r="T15" t="s">
@@ -37625,7 +38614,7 @@
       <c r="D16" t="str">
         <v>ES</v>
       </c>
-      <c r="S16" s="72" t="s">
+      <c r="S16" s="71" t="s">
         <v>113</v>
       </c>
       <c r="T16" t="s">
@@ -37647,7 +38636,7 @@
       <c r="D17" t="str">
         <v>RS</v>
       </c>
-      <c r="S17" s="72" t="s">
+      <c r="S17" s="71" t="s">
         <v>122</v>
       </c>
       <c r="T17" t="s">
@@ -37669,7 +38658,7 @@
       <c r="D18" t="str">
         <v>PR</v>
       </c>
-      <c r="S18" s="72" t="s">
+      <c r="S18" s="71" t="s">
         <v>589</v>
       </c>
       <c r="T18" t="s">
@@ -37691,7 +38680,7 @@
       <c r="D19" t="str">
         <v>AC</v>
       </c>
-      <c r="S19" s="72" t="s">
+      <c r="S19" s="71" t="s">
         <v>586</v>
       </c>
       <c r="T19" t="s">
@@ -37713,7 +38702,7 @@
       <c r="D20" t="str">
         <v>MT</v>
       </c>
-      <c r="S20" s="72" t="s">
+      <c r="S20" s="71" t="s">
         <v>91</v>
       </c>
       <c r="T20" t="s">
@@ -37735,7 +38724,7 @@
       <c r="D21" t="str">
         <v>RO</v>
       </c>
-      <c r="S21" s="72" t="s">
+      <c r="S21" s="71" t="s">
         <v>198</v>
       </c>
       <c r="T21" t="s">
@@ -37754,7 +38743,7 @@
       <c r="C22" t="str">
         <v>BARRA DOS COQUEIROS</v>
       </c>
-      <c r="S22" s="72" t="s">
+      <c r="S22" s="71" t="s">
         <v>569</v>
       </c>
       <c r="T22" t="s">
@@ -37773,7 +38762,7 @@
       <c r="C23" t="str">
         <v>CRATO</v>
       </c>
-      <c r="S23" s="72" t="s">
+      <c r="S23" s="71" t="s">
         <v>759</v>
       </c>
       <c r="T23" t="s">
@@ -37792,7 +38781,7 @@
       <c r="C24" t="str">
         <v>ITAPIPOCA</v>
       </c>
-      <c r="S24" s="72" t="s">
+      <c r="S24" s="71" t="s">
         <v>760</v>
       </c>
       <c r="T24" t="s">
@@ -37811,7 +38800,7 @@
       <c r="C25" t="str">
         <v>TAUÁ</v>
       </c>
-      <c r="S25" s="72" t="s">
+      <c r="S25" s="71" t="s">
         <v>761</v>
       </c>
       <c r="T25" t="s">
@@ -37830,7 +38819,7 @@
       <c r="C26" t="str">
         <v>BALSAS</v>
       </c>
-      <c r="S26" s="72" t="s">
+      <c r="S26" s="71" t="s">
         <v>116</v>
       </c>
       <c r="T26" t="s">
@@ -37849,7 +38838,7 @@
       <c r="C27" t="str">
         <v>MONTES CLAROS</v>
       </c>
-      <c r="S27" s="72" t="s">
+      <c r="S27" s="71" t="s">
         <v>119</v>
       </c>
       <c r="T27" t="s">
@@ -37868,7 +38857,7 @@
       <c r="C28" t="str">
         <v>ITATIAIA</v>
       </c>
-      <c r="S28" s="72" t="s">
+      <c r="S28" s="71" t="s">
         <v>762</v>
       </c>
       <c r="T28" t="s">
@@ -37887,7 +38876,7 @@
       <c r="C29" t="str">
         <v>COLATINA</v>
       </c>
-      <c r="S29" s="72" t="s">
+      <c r="S29" s="71" t="s">
         <v>763</v>
       </c>
       <c r="T29" t="s">
@@ -37906,7 +38895,7 @@
       <c r="C30" t="str">
         <v>VARGEM GRANDE</v>
       </c>
-      <c r="S30" s="72" t="s">
+      <c r="S30" s="71" t="s">
         <v>764</v>
       </c>
       <c r="T30" t="s">
@@ -37914,7 +38903,7 @@
       </c>
       <c r="U30" s="3">
         <f>COUNTIF(AREAS!L:L,Planilha2!T30)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V30" s="3">
         <f>_xlfn.XLOOKUP(T30,AREAS!L:L,AREAS!D:D,"não")</f>
@@ -37925,7 +38914,7 @@
       <c r="C31" t="str">
         <v>DUQUE DE CAXIAS</v>
       </c>
-      <c r="S31" s="72" t="s">
+      <c r="S31" s="71" t="s">
         <v>573</v>
       </c>
       <c r="T31" t="s">
@@ -37944,7 +38933,7 @@
       <c r="C32" t="str">
         <v>LUZIMANGUES</v>
       </c>
-      <c r="S32" s="72" t="s">
+      <c r="S32" s="71" t="s">
         <v>186</v>
       </c>
       <c r="T32" t="s">
@@ -37963,7 +38952,7 @@
       <c r="C33" t="str">
         <v>ITABORAÍ</v>
       </c>
-      <c r="S33" s="72" t="s">
+      <c r="S33" s="71" t="s">
         <v>180</v>
       </c>
       <c r="T33" t="s">
@@ -37982,7 +38971,7 @@
       <c r="C34" t="str">
         <v>MACAE</v>
       </c>
-      <c r="S34" s="72" t="s">
+      <c r="S34" s="71" t="s">
         <v>182</v>
       </c>
       <c r="T34" t="s">
@@ -38001,7 +38990,7 @@
       <c r="C35" t="str">
         <v>ARRAIAL DO CABO</v>
       </c>
-      <c r="S35" s="72" t="s">
+      <c r="S35" s="71" t="s">
         <v>765</v>
       </c>
       <c r="T35" t="s">
@@ -38020,7 +39009,7 @@
       <c r="C36" t="str">
         <v xml:space="preserve">PARAUAPEBAS </v>
       </c>
-      <c r="S36" s="72" t="s">
+      <c r="S36" s="71" t="s">
         <v>766</v>
       </c>
       <c r="T36" t="s">
@@ -38039,16 +39028,16 @@
       <c r="C37" t="str">
         <v xml:space="preserve">PORANGATU </v>
       </c>
-      <c r="S37" s="72" t="s">
+      <c r="S37" s="71" t="s">
         <v>196</v>
       </c>
-      <c r="T37" s="69" t="s">
+      <c r="T37" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="U37" s="70">
-        <v>1</v>
-      </c>
-      <c r="V37" s="70">
+      <c r="U37" s="69">
+        <v>1</v>
+      </c>
+      <c r="V37" s="69">
         <f>_xlfn.XLOOKUP(T37,AREAS!L:L,AREAS!D:D,"não")</f>
         <v>1</v>
       </c>
@@ -38057,7 +39046,7 @@
       <c r="C38" t="str">
         <v>LORENA</v>
       </c>
-      <c r="S38" s="72" t="s">
+      <c r="S38" s="71" t="s">
         <v>767</v>
       </c>
       <c r="T38" t="s">
@@ -38076,7 +39065,7 @@
       <c r="C39" t="str">
         <v>PRESIDENTE PRUDENTE</v>
       </c>
-      <c r="S39" s="72" t="s">
+      <c r="S39" s="71" t="s">
         <v>768</v>
       </c>
       <c r="T39" t="s">
@@ -38095,7 +39084,7 @@
       <c r="C40" t="str">
         <v>CAÇAPAVA</v>
       </c>
-      <c r="S40" s="72" t="s">
+      <c r="S40" s="71" t="s">
         <v>769</v>
       </c>
       <c r="T40" t="s">
@@ -38114,7 +39103,7 @@
       <c r="C41" t="str">
         <v>AVARÉ</v>
       </c>
-      <c r="S41" s="72" t="s">
+      <c r="S41" s="71" t="s">
         <v>57</v>
       </c>
       <c r="T41" t="s">
@@ -38133,7 +39122,7 @@
       <c r="C42" t="str">
         <v>RIO GRANDE DO SUL</v>
       </c>
-      <c r="S42" s="72" t="s">
+      <c r="S42" s="71" t="s">
         <v>29</v>
       </c>
       <c r="T42" t="s">
@@ -38152,7 +39141,7 @@
       <c r="C43" t="str">
         <v>POÇOS DE CALDAS</v>
       </c>
-      <c r="S43" s="72" t="s">
+      <c r="S43" s="71" t="s">
         <v>770</v>
       </c>
       <c r="T43" t="s">
@@ -38171,7 +39160,7 @@
       <c r="C44" t="str">
         <v>RIO DE JANEIRO</v>
       </c>
-      <c r="S44" s="72" t="s">
+      <c r="S44" s="71" t="s">
         <v>39</v>
       </c>
       <c r="T44" t="s">
@@ -38190,7 +39179,7 @@
       <c r="C45" t="str">
         <v>CABO FRIO</v>
       </c>
-      <c r="S45" s="72" t="s">
+      <c r="S45" s="71" t="s">
         <v>49</v>
       </c>
       <c r="T45" t="s">
@@ -38209,7 +39198,7 @@
       <c r="C46" t="str">
         <v>CACHOEIRA DO SUL</v>
       </c>
-      <c r="S46" s="72" t="s">
+      <c r="S46" s="71" t="s">
         <v>42</v>
       </c>
       <c r="T46" t="s">
@@ -38228,7 +39217,7 @@
       <c r="C47" t="str">
         <v>GUAÍBA</v>
       </c>
-      <c r="S47" s="72" t="s">
+      <c r="S47" s="71" t="s">
         <v>771</v>
       </c>
       <c r="T47" t="s">
@@ -38247,7 +39236,7 @@
       <c r="C48" t="str">
         <v>PORTO ALEGRE</v>
       </c>
-      <c r="S48" s="72" t="s">
+      <c r="S48" s="71" t="s">
         <v>772</v>
       </c>
       <c r="T48" t="s">
@@ -38266,7 +39255,7 @@
       <c r="C49" t="str">
         <v>SANTA CRUZ DO SUL</v>
       </c>
-      <c r="S49" s="72" t="s">
+      <c r="S49" s="71" t="s">
         <v>47</v>
       </c>
       <c r="T49" t="s">
@@ -38285,7 +39274,7 @@
       <c r="C50" t="str">
         <v>SÃO LEOPOLDO</v>
       </c>
-      <c r="S50" s="72" t="s">
+      <c r="S50" s="71" t="s">
         <v>172</v>
       </c>
       <c r="T50" t="s">
@@ -38304,7 +39293,7 @@
       <c r="C51" t="str">
         <v>CAXIAS DO SUL</v>
       </c>
-      <c r="S51" s="72" t="s">
+      <c r="S51" s="71" t="s">
         <v>173</v>
       </c>
       <c r="T51" t="s">
@@ -38323,7 +39312,7 @@
       <c r="C52" t="str">
         <v>CANELA</v>
       </c>
-      <c r="S52" s="72" t="s">
+      <c r="S52" s="71" t="s">
         <v>134</v>
       </c>
       <c r="T52" t="s">
@@ -38342,7 +39331,7 @@
       <c r="C53" t="str">
         <v>VIAMÃO</v>
       </c>
-      <c r="S53" s="72" t="s">
+      <c r="S53" s="71" t="s">
         <v>157</v>
       </c>
       <c r="T53" t="s">
@@ -38361,7 +39350,7 @@
       <c r="C54" t="str">
         <v>PELOTAS</v>
       </c>
-      <c r="S54" s="72" t="s">
+      <c r="S54" s="71" t="s">
         <v>127</v>
       </c>
       <c r="T54" t="s">
@@ -38380,7 +39369,7 @@
       <c r="C55" t="str">
         <v xml:space="preserve">UBERABA </v>
       </c>
-      <c r="S55" s="72" t="s">
+      <c r="S55" s="71" t="s">
         <v>130</v>
       </c>
       <c r="T55" t="s">
@@ -38399,7 +39388,7 @@
       <c r="C56" t="str">
         <v>VARZEA GRANDE</v>
       </c>
-      <c r="S56" s="72" t="s">
+      <c r="S56" s="71" t="s">
         <v>609</v>
       </c>
       <c r="T56" t="s">
@@ -38418,7 +39407,7 @@
       <c r="C57" t="str">
         <v>ALVORADA</v>
       </c>
-      <c r="S57" s="72" t="s">
+      <c r="S57" s="71" t="s">
         <v>773</v>
       </c>
       <c r="T57" t="s">
@@ -38437,7 +39426,7 @@
       <c r="C58" t="str">
         <v>SAPIRANGA</v>
       </c>
-      <c r="S58" s="72" t="s">
+      <c r="S58" s="71" t="s">
         <v>154</v>
       </c>
       <c r="T58" t="s">
@@ -38456,7 +39445,7 @@
       <c r="C59" t="str">
         <v>TORRES</v>
       </c>
-      <c r="S59" s="72" t="s">
+      <c r="S59" s="71" t="s">
         <v>774</v>
       </c>
       <c r="T59" t="s">
@@ -38475,7 +39464,7 @@
       <c r="C60" t="str">
         <v>GUARAPUAVA</v>
       </c>
-      <c r="S60" s="72" t="s">
+      <c r="S60" s="71" t="s">
         <v>775</v>
       </c>
       <c r="T60" t="s">
@@ -38494,7 +39483,7 @@
       <c r="C61" t="str">
         <v>VITORINO</v>
       </c>
-      <c r="S61" s="72" t="s">
+      <c r="S61" s="71" t="s">
         <v>776</v>
       </c>
       <c r="T61" t="s">
@@ -38513,7 +39502,7 @@
       <c r="C62" t="str">
         <v>RIO BRANCO</v>
       </c>
-      <c r="S62" s="72" t="s">
+      <c r="S62" s="71" t="s">
         <v>193</v>
       </c>
       <c r="T62" t="s">
@@ -38532,7 +39521,7 @@
       <c r="C63" t="str">
         <v>CÁCERES</v>
       </c>
-      <c r="S63" s="72" t="s">
+      <c r="S63" s="71" t="s">
         <v>187</v>
       </c>
       <c r="T63" t="s">
@@ -38551,7 +39540,7 @@
       <c r="C64" t="str">
         <v>TANGARÁ DA SERRA</v>
       </c>
-      <c r="S64" s="72" t="s">
+      <c r="S64" s="71" t="s">
         <v>189</v>
       </c>
       <c r="T64" t="s">
@@ -38570,7 +39559,7 @@
       <c r="C65" t="str">
         <v>CUIABÁ</v>
       </c>
-      <c r="S65" s="72" t="s">
+      <c r="S65" s="71" t="s">
         <v>565</v>
       </c>
       <c r="T65" t="s">
@@ -38589,7 +39578,7 @@
       <c r="C66" t="str">
         <v>CACOAL</v>
       </c>
-      <c r="S66" s="72" t="s">
+      <c r="S66" s="71" t="s">
         <v>191</v>
       </c>
       <c r="T66" t="s">
@@ -38608,7 +39597,7 @@
       <c r="C67" t="str">
         <v>JI-PARANÁ</v>
       </c>
-      <c r="S67" s="72" t="s">
+      <c r="S67" s="71" t="s">
         <v>169</v>
       </c>
       <c r="T67" t="s">
@@ -38627,7 +39616,7 @@
       <c r="C68" t="str">
         <v>ROLIM DE MOURA</v>
       </c>
-      <c r="S68" s="72" t="s">
+      <c r="S68" s="71" t="s">
         <v>159</v>
       </c>
       <c r="T68" t="s">
@@ -38646,7 +39635,7 @@
       <c r="C69" t="str">
         <v>ARIQUEMES</v>
       </c>
-      <c r="S69" s="72" t="s">
+      <c r="S69" s="71" t="s">
         <v>165</v>
       </c>
       <c r="T69" t="s">
@@ -38665,7 +39654,7 @@
       <c r="C70" t="str">
         <v>BELA VISTA DE GOIÁS</v>
       </c>
-      <c r="S70" s="72" t="s">
+      <c r="S70" s="71" t="s">
         <v>164</v>
       </c>
       <c r="T70" t="s">
@@ -38684,7 +39673,7 @@
       <c r="C71" t="str">
         <v>CONCEIÇÃO DO ARAGUAIA</v>
       </c>
-      <c r="S71" s="72" t="s">
+      <c r="S71" s="71" t="s">
         <v>160</v>
       </c>
       <c r="T71" t="s">
@@ -38703,7 +39692,7 @@
       <c r="C72" t="str">
         <v>GOIÂNIA</v>
       </c>
-      <c r="S72" s="72" t="s">
+      <c r="S72" s="71" t="s">
         <v>167</v>
       </c>
       <c r="T72" t="s">
@@ -38722,7 +39711,7 @@
       <c r="C73" t="str">
         <v>PORTO VELHO</v>
       </c>
-      <c r="S73" s="72" t="s">
+      <c r="S73" s="71" t="s">
         <v>161</v>
       </c>
       <c r="T73" t="s">
@@ -38741,7 +39730,7 @@
       <c r="C74" t="str">
         <v xml:space="preserve">XEREM </v>
       </c>
-      <c r="S74" s="72" t="s">
+      <c r="S74" s="71" t="s">
         <v>777</v>
       </c>
       <c r="T74" t="s">
@@ -38760,7 +39749,7 @@
       <c r="C75" t="str">
         <v>NOVO GAMA</v>
       </c>
-      <c r="S75" s="72" t="s">
+      <c r="S75" s="71" t="s">
         <v>162</v>
       </c>
       <c r="T75" t="s">
@@ -38779,7 +39768,7 @@
       <c r="C76" t="str">
         <v>CHAPADA DOS GUIMARÃES</v>
       </c>
-      <c r="S76" s="72" t="s">
+      <c r="S76" s="71" t="s">
         <v>170</v>
       </c>
       <c r="T76" t="s">
@@ -38798,7 +39787,7 @@
       <c r="C77" t="str">
         <v>CALDAS NOVAS</v>
       </c>
-      <c r="S77" s="72" t="s">
+      <c r="S77" s="71" t="s">
         <v>163</v>
       </c>
       <c r="T77" t="s">
@@ -38814,76 +39803,76 @@
       </c>
     </row>
     <row r="78" spans="3:22" x14ac:dyDescent="0.35">
-      <c r="S78" s="72" t="s">
+      <c r="S78" s="71" t="s">
         <v>171</v>
       </c>
       <c r="U78" s="3">
         <f>SUM(U6:U77)</f>
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="79" spans="3:22" x14ac:dyDescent="0.35">
-      <c r="S79" s="72" t="s">
+      <c r="S79" s="71" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="80" spans="3:22" x14ac:dyDescent="0.35">
-      <c r="S80" s="72" t="s">
+      <c r="S80" s="71" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="81" spans="19:19" x14ac:dyDescent="0.35">
-      <c r="S81" s="72" t="s">
+      <c r="S81" s="71" t="s">
         <v>778</v>
       </c>
     </row>
     <row r="82" spans="19:19" x14ac:dyDescent="0.35">
-      <c r="S82" s="72" t="s">
+      <c r="S82" s="71" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="83" spans="19:19" x14ac:dyDescent="0.35">
-      <c r="S83" s="72" t="s">
+      <c r="S83" s="71" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="84" spans="19:19" x14ac:dyDescent="0.35">
-      <c r="S84" s="72" t="s">
+      <c r="S84" s="71" t="s">
         <v>779</v>
       </c>
     </row>
     <row r="85" spans="19:19" x14ac:dyDescent="0.35">
-      <c r="S85" s="72" t="s">
+      <c r="S85" s="71" t="s">
         <v>611</v>
       </c>
     </row>
     <row r="86" spans="19:19" x14ac:dyDescent="0.35">
-      <c r="S86" s="72" t="s">
+      <c r="S86" s="71" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="87" spans="19:19" x14ac:dyDescent="0.35">
-      <c r="S87" s="72" t="s">
+      <c r="S87" s="71" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="88" spans="19:19" x14ac:dyDescent="0.35">
-      <c r="S88" s="72" t="s">
+      <c r="S88" s="71" t="s">
         <v>780</v>
       </c>
     </row>
     <row r="89" spans="19:19" x14ac:dyDescent="0.35">
-      <c r="S89" s="72" t="s">
+      <c r="S89" s="71" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="90" spans="19:19" x14ac:dyDescent="0.35">
-      <c r="S90" s="72" t="s">
+      <c r="S90" s="71" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="91" spans="19:19" x14ac:dyDescent="0.35">
-      <c r="S91" s="72" t="s">
+      <c r="S91" s="71" t="s">
         <v>781</v>
       </c>
     </row>

</xml_diff>